<commit_message>
Added more edge summaries for Addiction in Anatomy of the 42
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="423" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA47FF1C-0053-4C7D-A614-AE4B7C266E48}"/>
+  <xr:revisionPtr revIDLastSave="429" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF2A1B7-21F5-4069-ADB5-C09BFBCA7EB4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -3705,7 +3705,7 @@
         <v>Edu: Quality</v>
       </c>
       <c r="B14" s="24">
-        <v>-0.13</v>
+        <v>-0.17</v>
       </c>
       <c r="C14" s="23">
         <v>0.12</v>
@@ -3847,7 +3847,7 @@
         <v>Employment</v>
       </c>
       <c r="B15" s="24">
-        <v>-0.18</v>
+        <v>-0.23</v>
       </c>
       <c r="C15" s="23">
         <v>0.24</v>
@@ -4131,10 +4131,10 @@
         <v>Equality</v>
       </c>
       <c r="B17" s="24">
-        <v>-0.06</v>
+        <v>-0.11</v>
       </c>
       <c r="C17" s="23">
-        <v>-0.11</v>
+        <v>-0.09</v>
       </c>
       <c r="D17" s="24">
         <v>-7.0000000000000007E-2</v>
@@ -9861,7 +9861,7 @@
     </customSheetView>
   </customSheetViews>
   <conditionalFormatting sqref="A2:XFD2">
-    <cfRule type="colorScale" priority="12">
+    <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9873,6 +9873,338 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:XFD37 A40:XFD43">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:XFD4">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A6:XFD6">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A7:XFD7">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A8:XFD8">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A9:XFD9">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A10:XFD10">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A24:XFD24 M26">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A34:XFD34">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A35:XFD35">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A38:XFD38">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A39:XFD39">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2 B26:Y26">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:AQ37 B40:AQ43">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7:AQ7">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I8:XFD8 A8:G8 G6:XFD6 A6:E6 E4:XFD4 A4:C4 C2:XFD2 A2 J9:XFD9 A9:H9 K10:XFD10 A10:I10 N13:XFD13 A13:L13 W22:XFD22 A22:U22 Y24:XFD24 A24:W24 AI34:XFD34 A34:AG34 AJ35:XFD35 A35:AH35">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL38 AM39">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO40:AP40 AP41 O14:AK14 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 O19:R19 T21 T22:U22 T23:V23 T24:W24 Z27 Z28:AA28 Z29:AB29 Z30:AC30 Z31:AD31 Z32:AE32 Z33:AF33 Z34:AG34 Z35:AH35 Z36:AI36 Z37:AJ37 Z40:AM40 Z41:AN41 Z42:AO42 Z43:AP43 G8:G12 T25:X25 O20:S25 F2:L3 E4:F4 AQ14:AQ32 H7:K7 L7:L11 G4:L6 AM24:AP28 P15:AK15 Q16:AK16 R17:AK17 S18:AK18 T19:AK19 U20:AK20 V21:AK21 W22:AK22 X23:AK23 Y24:AL24 Z25:AL25 AA26:AL26 AB27:AL27 AC28:AL28 AD29:AP29 AE30:AP30 AF31:AP31 AG32:AP32 AQ34:AQ37 AH33:AQ33 AI34:AP34 AJ35:AP35 AK36:AP36 AL37:AP37 AQ40:AQ42 N13:AK13 M2:AQ12 AN13:AQ13 AN14:AP23 AL13:AM23 M15:N25 M14 H11:J11 H12:K12 H35:Y37 L24:L25 H24:K34 G24:G37 G13:L23 F7:F16 D6:E16 D17:F37 D5 B4:C37 L26:Y34 B40:Y43">
+    <cfRule type="colorScale" priority="215">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 D46:E46 B46 C45:E45 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 F45:M46 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N45:AQ56 AL57:AP67 O69:Y70 K60:N70">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 X24 W23 V22 U21 T20 S19 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2">
+    <cfRule type="colorScale" priority="43">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR43:XFD43 A43:AP43 AQ42:XFD42 A42:AO42 AP41:XFD41 A41:AN41 AO40:XFD40 A40:AM40 AL37:XFD37 A37:AJ37 AK36:XFD36 A36:AI36 AJ35:XFD35 A35:AH35 AI34:XFD34 A34:AG34 AH33:XFD33 A33:AF33 AG32:XFD32 A32:AE32 AF31:XFD31 A31:AD31 AE30:XFD30 A30:AC30 AD29:XFD29 A29:AB29 AC28:XFD28 A28:AA28 AB27:XFD27 A27:Z27 AA26:XFD26 Z25:XFD25 A25:X25 Y24:XFD24 A24:W24 X23:XFD23 A23:V23 W22:XFD22 A22:U22 V21:XFD21 A21:T21 U20:XFD20 A20:S20 T19:XFD19 A19:R19 S18:XFD18 A18:Q18 R17:XFD17 A17:P17 Q16:XFD16 A16:O16 P15:XFD15 A15:N15 O14:XFD14 A14:M14 N13:XFD13 A13:L13 M12:XFD12 A12:K12 L11:XFD11 A11:J11 K10:XFD10 A10:I10 J9:XFD9 A9:H9 I8:XFD8 A8:G8 H7:XFD7 A7:F7 G6:XFD6 A6:E6 F5:XFD5 A5:D5 E4:XFD4 A4:C4 D3:XFD3 A3:B3 C2:XFD2 A2 A26:Y26">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -9884,140 +10216,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:XFD4">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6:XFD6">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A7:XFD7">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A8:XFD8">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A9:XFD9">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A10:XFD10">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A24:XFD24 M26">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A34:XFD34">
-    <cfRule type="colorScale" priority="24">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A35:XFD35">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A38:XFD38">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A39:XFD39">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2">
-    <cfRule type="colorScale" priority="11">
+  <conditionalFormatting sqref="G7">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10025,194 +10225,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2 B26:Y26">
-    <cfRule type="colorScale" priority="25">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AQ37 B40:AQ43">
-    <cfRule type="colorScale" priority="27">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I8:XFD8 A8:G8 G6:XFD6 A6:E6 E4:XFD4 A4:C4 C2:XFD2 A2 J9:XFD9 A9:H9 K10:XFD10 A10:I10 N13:XFD13 A13:L13 W22:XFD22 A22:U22 Y24:XFD24 A24:W24 AI34:XFD34 A34:AG34 AJ35:XFD35 A35:AH35">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="44">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="32">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO40:AP40 AP41 O14:AK14 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 O19:R19 T21 T22:U22 T23:V23 T24:W24 Z27 Z28:AA28 Z29:AB29 Z30:AC30 Z31:AD31 Z32:AE32 Z33:AF33 Z34:AG34 Z35:AH35 Z36:AI36 Z37:AJ37 Z40:AM40 Z41:AN41 Z42:AO42 Z43:AP43 G8:G12 T25:X25 O20:S25 F2:L3 E4:F4 AQ14:AQ32 H7:K7 L7:L11 G4:L6 AM24:AP28 P15:AK15 Q16:AK16 R17:AK17 S18:AK18 T19:AK19 U20:AK20 V21:AK21 W22:AK22 X23:AK23 Y24:AL24 Z25:AL25 AA26:AL26 AB27:AL27 AC28:AL28 AD29:AP29 AE30:AP30 AF31:AP31 AG32:AP32 AQ34:AQ37 AH33:AQ33 AI34:AP34 AJ35:AP35 AK36:AP36 AL37:AP37 AQ40:AQ42 N13:AK13 M2:AQ12 AN13:AQ13 AN14:AP23 AL13:AM23 M15:N25 M14 H11:J11 H12:K12 H35:Y37 L24:L25 H24:K34 G24:G37 G13:L23 F7:F16 D6:E16 D17:F37 D5 B4:C37 L26:Y34 B40:Y43">
-    <cfRule type="colorScale" priority="214">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 D46:E46 B46 C45:E45 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 F45:M46 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N45:AQ56 AL57:AP67 O69:Y70 K60:N70">
-    <cfRule type="colorScale" priority="29">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 X24 W23 V22 U21 T20 S19 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2">
-    <cfRule type="colorScale" priority="42">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="43">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AR43:XFD43 A43:AP43 AQ42:XFD42 A42:AO42 AP41:XFD41 A41:AN41 AO40:XFD40 A40:AM40 AL37:XFD37 A37:AJ37 AK36:XFD36 A36:AI36 AJ35:XFD35 A35:AH35 AI34:XFD34 A34:AG34 AH33:XFD33 A33:AF33 AG32:XFD32 A32:AE32 AF31:XFD31 A31:AD31 AE30:XFD30 A30:AC30 AD29:XFD29 A29:AB29 AC28:XFD28 A28:AA28 AB27:XFD27 A27:Z27 AA26:XFD26 Z25:XFD25 A25:X25 Y24:XFD24 A24:W24 X23:XFD23 A23:V23 W22:XFD22 A22:U22 V21:XFD21 A21:T21 U20:XFD20 A20:S20 T19:XFD19 A19:R19 S18:XFD18 A18:Q18 R17:XFD17 A17:P17 Q16:XFD16 A16:O16 P15:XFD15 A15:N15 O14:XFD14 A14:M14 N13:XFD13 A13:L13 M12:XFD12 A12:K12 L11:XFD11 A11:J11 K10:XFD10 A10:I10 J9:XFD9 A9:H9 I8:XFD8 A8:G8 H7:XFD7 A7:F7 G6:XFD6 A6:E6 F5:XFD5 A5:D5 E4:XFD4 A4:C4 D3:XFD3 A3:B3 C2:XFD2 A2 A26:Y26">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B7:AQ7">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10519,7 +10531,7 @@
       </c>
       <c r="D13" s="35">
         <f>'Influence Matrix'!B14</f>
-        <v>-0.13</v>
+        <v>-0.17</v>
       </c>
       <c r="G13" t="s">
         <v>78</v>
@@ -10540,7 +10552,7 @@
       </c>
       <c r="D14" s="35">
         <f>'Influence Matrix'!B15</f>
-        <v>-0.18</v>
+        <v>-0.23</v>
       </c>
       <c r="G14" t="s">
         <v>78</v>
@@ -10582,7 +10594,7 @@
       </c>
       <c r="D16" s="35">
         <f>'Influence Matrix'!B17</f>
-        <v>-0.06</v>
+        <v>-0.11</v>
       </c>
       <c r="G16" t="s">
         <v>125</v>
@@ -11365,7 +11377,7 @@
       </c>
       <c r="D57" s="44">
         <f>'Influence Matrix'!C17</f>
-        <v>-0.11</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Minor update to Addiction repo, added research and finished notes/text docs for 'gun rights' and 'healthcare access'; changed document filenames to stable convention; minore touch-ups for README
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="429" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF2A1B7-21F5-4069-ADB5-C09BFBCA7EB4}"/>
+  <xr:revisionPtr revIDLastSave="430" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53EA85F6-FB8C-4B33-BBE1-344F33ADC538}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -4557,7 +4557,7 @@
         <v>Gun Rights</v>
       </c>
       <c r="B20" s="24">
-        <v>-0.12</v>
+        <v>-0.06</v>
       </c>
       <c r="C20" s="23">
         <v>0.01</v>
@@ -10016,7 +10016,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -10028,7 +10028,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
     <cfRule type="colorScale" priority="45">
       <colorScale>
         <cfvo type="min"/>
@@ -10052,7 +10052,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
     <cfRule type="colorScale" priority="33">
       <colorScale>
         <cfvo type="min"/>
@@ -10100,8 +10100,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
     <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10124,7 +10136,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
+  <conditionalFormatting sqref="AM39 AL38">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -10216,18 +10228,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G7">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="90" orientation="portrait" horizontalDpi="4294967293" r:id="rId2"/>
 </worksheet>
@@ -10660,7 +10660,7 @@
       </c>
       <c r="D19" s="35">
         <f>'Influence Matrix'!B20</f>
-        <v>-0.12</v>
+        <v>-0.06</v>
       </c>
       <c r="G19" t="s">
         <v>78</v>

</xml_diff>

<commit_message>
Repo: Added a note about higher-order curve shaping to notes/model_extensions/; Research Repo: completed notes.txt and links.txt for add_heac and add_heaq; Anotomy of the 42: updated addiction edge summaries
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="430" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53EA85F6-FB8C-4B33-BBE1-344F33ADC538}"/>
+  <xr:revisionPtr revIDLastSave="432" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53DAC913-1A05-4228-B4C1-1B0E0D331439}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -4841,7 +4841,7 @@
         <v>HC Cost</v>
       </c>
       <c r="B22" s="24">
-        <v>0.17</v>
+        <v>0.32</v>
       </c>
       <c r="C22" s="23">
         <v>0.11</v>
@@ -4983,7 +4983,7 @@
         <v>HC Quality</v>
       </c>
       <c r="B23" s="24">
-        <v>-0.14000000000000001</v>
+        <v>-0.15</v>
       </c>
       <c r="C23" s="23">
         <v>-7.0000000000000007E-2</v>
@@ -10702,7 +10702,7 @@
       </c>
       <c r="D21" s="35">
         <f>'Influence Matrix'!B22</f>
-        <v>0.17</v>
+        <v>0.32</v>
       </c>
       <c r="G21" t="s">
         <v>85</v>
@@ -10723,7 +10723,7 @@
       </c>
       <c r="D22" s="35">
         <f>'Influence Matrix'!B23</f>
-        <v>-0.14000000000000001</v>
+        <v>-0.15</v>
       </c>
       <c r="G22" t="s">
         <v>78</v>

</xml_diff>

<commit_message>
Finished Research Repo influences for: add_inf, add_inn, add_lawe, and add_lib
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="565" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F010EC87-88DD-4827-952A-42CB4D61FE67}"/>
+  <xr:revisionPtr revIDLastSave="567" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4890BED3-2225-4063-96B9-1F746CAE3AA0}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -1253,7 +1253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1366,6 +1366,22 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1392,31 +1408,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5707,7 +5698,7 @@
         <v>Law Enforcement</v>
       </c>
       <c r="B28" s="13">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="C28" s="12">
         <v>-0.09</v>
@@ -5849,7 +5840,7 @@
         <v>Liberty</v>
       </c>
       <c r="B29" s="13">
-        <v>-0.21</v>
+        <v>-0.22</v>
       </c>
       <c r="C29" s="12">
         <v>0.25</v>
@@ -10030,30 +10021,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B2">
     <cfRule type="colorScale" priority="12">
       <colorScale>
@@ -10063,18 +10030,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10114,7 +10069,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
+  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -10150,7 +10117,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
+  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39 AL38">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -10842,7 +10833,7 @@
       </c>
       <c r="D27" s="24">
         <f>'Influence Matrix'!B28</f>
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="G27" t="s">
         <v>72</v>
@@ -10863,7 +10854,7 @@
       </c>
       <c r="D28" s="24">
         <f>'Influence Matrix'!B29</f>
-        <v>-0.21</v>
+        <v>-0.22</v>
       </c>
       <c r="G28" t="s">
         <v>72</v>
@@ -11825,7 +11816,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6229F6B-4F53-41D8-AF16-43616E62B79A}">
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
@@ -11838,404 +11829,205 @@
     <col min="8" max="8" width="115.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>26</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="57"/>
-      <c r="O2" s="57"/>
-    </row>
-    <row r="3" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>38</v>
       </c>
       <c r="B3" s="1"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-    </row>
-    <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="1"/>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="52" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="47"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="60"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="57"/>
-      <c r="O4" s="57"/>
-    </row>
-    <row r="5" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D4" s="53"/>
+      <c r="J4" s="46"/>
+      <c r="K4" s="46"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="46"/>
+    </row>
+    <row r="5" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="1"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="49"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
-      <c r="M5" s="59"/>
-      <c r="N5" s="57"/>
-      <c r="O5" s="57"/>
-    </row>
-    <row r="6" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="54"/>
+      <c r="D5" s="55"/>
+    </row>
+    <row r="6" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>35</v>
       </c>
       <c r="B6" s="1"/>
-      <c r="C6" s="50"/>
-      <c r="D6" s="51"/>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59"/>
-      <c r="K6" s="59"/>
-      <c r="L6" s="59"/>
-      <c r="M6" s="59"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="57"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="C6" s="56"/>
+      <c r="D6" s="57"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="1"/>
-      <c r="I7" s="59"/>
-      <c r="J7" s="59"/>
-      <c r="K7" s="59"/>
-      <c r="L7" s="59"/>
-      <c r="M7" s="59"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="1"/>
-      <c r="I8" s="59"/>
-      <c r="J8" s="59"/>
-      <c r="K8" s="59"/>
-      <c r="L8" s="59"/>
-      <c r="M8" s="59"/>
-      <c r="N8" s="57"/>
-      <c r="O8" s="57"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>46</v>
       </c>
       <c r="B9" s="1"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
-      <c r="M9" s="59"/>
-      <c r="N9" s="57"/>
-      <c r="O9" s="57"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B10" s="1"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-      <c r="K10" s="59"/>
-      <c r="L10" s="59"/>
-      <c r="M10" s="59"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="57"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>30</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="59"/>
-      <c r="L11" s="59"/>
-      <c r="M11" s="59"/>
-      <c r="N11" s="57"/>
-      <c r="O11" s="57"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="I12" s="59"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="59"/>
-      <c r="L12" s="59"/>
-      <c r="M12" s="59"/>
-      <c r="N12" s="57"/>
-      <c r="O12" s="57"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="I13" s="59"/>
-      <c r="J13" s="59"/>
-      <c r="K13" s="59"/>
-      <c r="L13" s="59"/>
-      <c r="M13" s="59"/>
-      <c r="N13" s="57"/>
-      <c r="O13" s="57"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>5</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="I14" s="57"/>
-      <c r="J14" s="57"/>
-      <c r="K14" s="57"/>
-      <c r="L14" s="57"/>
-      <c r="M14" s="57"/>
-      <c r="N14" s="57"/>
-      <c r="O14" s="57"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>36</v>
       </c>
       <c r="B15" s="1"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="57"/>
-      <c r="L15" s="57"/>
-      <c r="M15" s="57"/>
-      <c r="N15" s="57"/>
-      <c r="O15" s="57"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>18</v>
       </c>
       <c r="B16" s="1"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="57"/>
-      <c r="L16" s="57"/>
-      <c r="M16" s="57"/>
-      <c r="N16" s="57"/>
-      <c r="O16" s="57"/>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>39</v>
       </c>
       <c r="B17" s="1"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="57"/>
-      <c r="L17" s="57"/>
-      <c r="M17" s="57"/>
-      <c r="N17" s="57"/>
-      <c r="O17" s="57"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>43</v>
       </c>
       <c r="B18" s="1"/>
-      <c r="F18" s="55"/>
-      <c r="I18" s="57"/>
-      <c r="J18" s="57"/>
-      <c r="K18" s="57"/>
-      <c r="L18" s="57"/>
-      <c r="M18" s="57"/>
-      <c r="N18" s="57"/>
-      <c r="O18" s="57"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B19" s="1"/>
-      <c r="F19" s="55"/>
-      <c r="I19" s="57"/>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57"/>
-      <c r="L19" s="57"/>
-      <c r="M19" s="57"/>
-      <c r="N19" s="57"/>
-      <c r="O19" s="57"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B20" s="1"/>
-      <c r="F20" s="56"/>
-      <c r="I20" s="57"/>
-      <c r="J20" s="57"/>
-      <c r="K20" s="57"/>
-      <c r="L20" s="57"/>
-      <c r="M20" s="57"/>
-      <c r="N20" s="57"/>
-      <c r="O20" s="57"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B21" s="1"/>
-      <c r="F21" s="56"/>
-      <c r="I21" s="57"/>
-      <c r="J21" s="57"/>
-      <c r="K21" s="57"/>
-      <c r="L21" s="57"/>
-      <c r="M21" s="57"/>
-      <c r="N21" s="57"/>
-      <c r="O21" s="57"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B22" s="1"/>
-      <c r="F22" s="56"/>
-      <c r="I22" s="57"/>
-      <c r="J22" s="57"/>
-      <c r="K22" s="57"/>
-      <c r="L22" s="57"/>
-      <c r="M22" s="57"/>
-      <c r="N22" s="57"/>
-      <c r="O22" s="57"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>6</v>
       </c>
       <c r="B23" s="1"/>
-      <c r="F23" s="56"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="57"/>
-      <c r="K23" s="57"/>
-      <c r="L23" s="57"/>
-      <c r="M23" s="57"/>
-      <c r="N23" s="57"/>
-      <c r="O23" s="57"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B24" s="1"/>
-      <c r="F24" s="55"/>
-      <c r="I24" s="57"/>
-      <c r="J24" s="57"/>
-      <c r="K24" s="57"/>
-      <c r="L24" s="57"/>
-      <c r="M24" s="57"/>
-      <c r="N24" s="57"/>
-      <c r="O24" s="57"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>8</v>
       </c>
       <c r="B25" s="1"/>
-      <c r="F25" s="55"/>
-      <c r="I25" s="57"/>
-      <c r="J25" s="57"/>
-      <c r="K25" s="57"/>
-      <c r="L25" s="57"/>
-      <c r="M25" s="57"/>
-      <c r="N25" s="57"/>
-      <c r="O25" s="57"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>9</v>
       </c>
       <c r="B26" s="1"/>
-      <c r="F26" s="55"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="57"/>
-      <c r="L26" s="57"/>
-      <c r="M26" s="57"/>
-      <c r="N26" s="57"/>
-      <c r="O26" s="57"/>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>148</v>
       </c>
       <c r="B27" s="1"/>
-      <c r="I27" s="57"/>
-      <c r="J27" s="57"/>
-      <c r="K27" s="57"/>
-      <c r="L27" s="57"/>
-      <c r="M27" s="57"/>
-      <c r="N27" s="57"/>
-      <c r="O27" s="57"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>10</v>
       </c>
       <c r="B28" s="1"/>
-      <c r="I28" s="57"/>
-      <c r="J28" s="57"/>
-      <c r="K28" s="57"/>
-      <c r="L28" s="57"/>
-      <c r="M28" s="57"/>
-      <c r="N28" s="57"/>
-      <c r="O28" s="57"/>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>11</v>
       </c>
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>164</v>
       </c>
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>12</v>
       </c>
@@ -12275,13 +12067,13 @@
         <v>45</v>
       </c>
       <c r="B37" s="32"/>
-      <c r="C37" s="52" t="s">
+      <c r="C37" s="58" t="s">
         <v>170</v>
       </c>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="52"/>
+      <c r="D37" s="58"/>
+      <c r="E37" s="58"/>
+      <c r="F37" s="58"/>
+      <c r="G37" s="58"/>
       <c r="H37" s="28"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -12289,11 +12081,11 @@
         <v>171</v>
       </c>
       <c r="B38" s="31"/>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="52"/>
-      <c r="F38" s="52"/>
-      <c r="G38" s="52"/>
+      <c r="C38" s="58"/>
+      <c r="D38" s="58"/>
+      <c r="E38" s="58"/>
+      <c r="F38" s="58"/>
+      <c r="G38" s="58"/>
       <c r="H38" s="28"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -12301,11 +12093,11 @@
         <v>17</v>
       </c>
       <c r="B39" s="25"/>
-      <c r="C39" s="52"/>
-      <c r="D39" s="52"/>
-      <c r="E39" s="52"/>
-      <c r="F39" s="52"/>
-      <c r="G39" s="52"/>
+      <c r="C39" s="58"/>
+      <c r="D39" s="58"/>
+      <c r="E39" s="58"/>
+      <c r="F39" s="58"/>
+      <c r="G39" s="58"/>
       <c r="H39" s="28"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -12313,11 +12105,11 @@
         <v>34</v>
       </c>
       <c r="B40" s="25"/>
-      <c r="C40" s="52"/>
-      <c r="D40" s="52"/>
-      <c r="E40" s="52"/>
-      <c r="F40" s="52"/>
-      <c r="G40" s="52"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="58"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="58"/>
+      <c r="G40" s="58"/>
       <c r="H40" s="28"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -12372,23 +12164,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="J2" s="64" t="s">
+      <c r="J2" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="K2" s="65"/>
+      <c r="K2" s="51"/>
     </row>
     <row r="3" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="53" t="s">
+      <c r="B3" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="54"/>
+      <c r="C3" s="60"/>
       <c r="E3" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="J3" s="61" t="s">
+      <c r="J3" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="K3" s="63" t="s">
+      <c r="K3" s="49" t="s">
         <v>178</v>
       </c>
     </row>
@@ -12400,10 +12192,10 @@
       <c r="E4" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="J4" s="62" t="s">
+      <c r="J4" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="63" t="s">
+      <c r="K4" s="49" t="s">
         <v>179</v>
       </c>
     </row>
@@ -12415,10 +12207,10 @@
       <c r="E5" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="J5" s="62" t="s">
+      <c r="J5" s="48" t="s">
         <v>55</v>
       </c>
-      <c r="K5" s="63" t="s">
+      <c r="K5" s="49" t="s">
         <v>180</v>
       </c>
     </row>
@@ -12430,10 +12222,10 @@
       <c r="E6" s="41" t="s">
         <v>165</v>
       </c>
-      <c r="J6" s="62" t="s">
+      <c r="J6" s="48" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="63" t="s">
+      <c r="K6" s="49" t="s">
         <v>181</v>
       </c>
     </row>
@@ -12441,10 +12233,10 @@
       <c r="E7" s="41" t="s">
         <v>166</v>
       </c>
-      <c r="J7" s="62" t="s">
+      <c r="J7" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="63" t="s">
+      <c r="K7" s="49" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12452,10 +12244,10 @@
       <c r="E8" s="41" t="s">
         <v>167</v>
       </c>
-      <c r="J8" s="62" t="s">
+      <c r="J8" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="63" t="s">
+      <c r="K8" s="49" t="s">
         <v>183</v>
       </c>
     </row>
@@ -12463,10 +12255,10 @@
       <c r="E9" s="41" t="s">
         <v>168</v>
       </c>
-      <c r="J9" s="62" t="s">
+      <c r="J9" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="K9" s="63" t="s">
+      <c r="K9" s="49" t="s">
         <v>184</v>
       </c>
     </row>
@@ -12474,68 +12266,68 @@
       <c r="E10" s="41" t="s">
         <v>169</v>
       </c>
-      <c r="J10" s="62" t="s">
+      <c r="J10" s="48" t="s">
         <v>56</v>
       </c>
-      <c r="K10" s="63" t="s">
+      <c r="K10" s="49" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="E11" s="41"/>
-      <c r="J11" s="62" t="s">
+      <c r="J11" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="K11" s="63" t="s">
+      <c r="K11" s="49" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="12" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E12" s="42"/>
-      <c r="J12" s="62" t="s">
+      <c r="J12" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="K12" s="63" t="s">
+      <c r="K12" s="49" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="J13" s="62" t="s">
+      <c r="J13" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="K13" s="63" t="s">
+      <c r="K13" s="49" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="J14" s="62" t="s">
+      <c r="J14" s="48" t="s">
         <v>60</v>
       </c>
-      <c r="K14" s="63" t="s">
+      <c r="K14" s="49" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="J15" s="62" t="s">
+      <c r="J15" s="48" t="s">
         <v>172</v>
       </c>
-      <c r="K15" s="63" t="s">
+      <c r="K15" s="49" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="J16" s="62" t="s">
+      <c r="J16" s="48" t="s">
         <v>173</v>
       </c>
-      <c r="K16" s="63" t="s">
+      <c r="K16" s="49" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="17" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J17" s="63" t="s">
+      <c r="J17" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="K17" s="63" t="s">
+      <c r="K17" s="49" t="s">
         <v>176</v>
       </c>
     </row>

</xml_diff>

<commit_message>
changed 'family values' to 'family orientation'; added addiction edges to 'Anatomy of the 42'
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="567" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4890BED3-2225-4063-96B9-1F746CAE3AA0}"/>
+  <xr:revisionPtr revIDLastSave="571" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DEBBE56-2892-42D7-B362-0956DA69F82B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -26,6 +26,7 @@
   <customWorkbookViews>
     <customWorkbookView name="ALL" guid="{C6883EF1-A235-4F7F-9B70-0CC3974E9739}" maximized="1" xWindow="1912" yWindow="126" windowWidth="1376" windowHeight="736" activeSheetId="1"/>
   </customWorkbookViews>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -68,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="191">
   <si>
     <t>Agriculture</t>
   </si>
@@ -638,6 +639,9 @@
   </si>
   <si>
     <t>degree to which social, political, and economic power is disproportionately held by men.</t>
+  </si>
+  <si>
+    <t>Family Orientation</t>
   </si>
 </sst>
 </file>
@@ -1911,7 +1915,7 @@
         <v>Equality</v>
       </c>
       <c r="R1" s="19" t="str">
-        <v>Family Values</v>
+        <v>Family Orientation</v>
       </c>
       <c r="S1" s="19" t="str">
         <v>Freedom of Speech</v>
@@ -4275,7 +4279,7 @@
     <row r="18" spans="1:53" ht="17.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="str">
         <f>Sliders!A17</f>
-        <v>Family Values</v>
+        <v>Family Orientation</v>
       </c>
       <c r="B18" s="13">
         <v>-0.21</v>
@@ -6692,7 +6696,7 @@
         <v>Poverty</v>
       </c>
       <c r="B35" s="13">
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="C35" s="12">
         <v>-0.24</v>
@@ -10021,6 +10025,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2">
     <cfRule type="colorScale" priority="12">
       <colorScale>
@@ -10030,6 +10058,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10069,19 +10109,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -10117,31 +10145,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM39 AL38">
+  <conditionalFormatting sqref="AL38 AM39">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -10980,7 +10984,7 @@
       </c>
       <c r="D34" s="24">
         <f>'Influence Matrix'!B35</f>
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="G34" t="s">
         <v>72</v>
@@ -11939,7 +11943,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>39</v>
+        <v>190</v>
       </c>
       <c r="B17" s="1"/>
     </row>

</xml_diff>

<commit_message>
commit 'Anatomy of the 42' v3.2.3; UPDATED MODEL ASSIGNMENTS: replaced 'Purpose/Meaning' variable with 'Rule of Law'
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="571" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DEBBE56-2892-42D7-B362-0956DA69F82B}"/>
+  <xr:revisionPtr revIDLastSave="586" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24DF861D-60B6-4391-8939-3299BC1E975D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="193">
   <si>
     <t>Agriculture</t>
   </si>
@@ -642,6 +642,12 @@
   </si>
   <si>
     <t>Family Orientation</t>
+  </si>
+  <si>
+    <t>Sense of Purpose/Meaing</t>
+  </si>
+  <si>
+    <t>Happiness</t>
   </si>
 </sst>
 </file>
@@ -1972,7 +1978,7 @@
         <v>Public Trust</v>
       </c>
       <c r="AK1" s="19" t="str">
-        <v>Purpose/Meaning</v>
+        <v>Rule of Law</v>
       </c>
       <c r="AL1" s="19" t="str">
         <v>Sickness/Disease</v>
@@ -6977,10 +6983,10 @@
     <row r="37" spans="1:53" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="str">
         <f>Sliders!A36</f>
-        <v>Purpose/Meaning</v>
+        <v>Rule of Law</v>
       </c>
       <c r="B37" s="13">
-        <v>-0.38</v>
+        <v>-0.17</v>
       </c>
       <c r="C37" s="12">
         <v>0.2</v>
@@ -7122,7 +7128,7 @@
         <v>Sickness/Disease</v>
       </c>
       <c r="B38" s="13">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="C38" s="12">
         <v>0.3</v>
@@ -9870,6 +9876,270 @@
     </customSheetView>
   </customSheetViews>
   <conditionalFormatting sqref="A2:XFD2">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:XFD37 A40:XFD43">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:XFD4">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A6:XFD6">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A7:XFD7">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A8:XFD8">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A9:XFD9">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A10:XFD10">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A24:XFD24 M26">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A34:XFD34">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A35:XFD35">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A38:XFD38">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A39:XFD39">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="38">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2 B26:Y26">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:AQ37 B40:AQ43">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7:AQ7">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I8:XFD8 A8:G8 G6:XFD6 A6:E6 E4:XFD4 A4:C4 C2:XFD2 A2 J9:XFD9 A9:H9 K10:XFD10 A10:I10 N13:XFD13 A13:L13 W22:XFD22 A22:U22 Y24:XFD24 A24:W24 AI34:XFD34 A34:AG34 AJ35:XFD35 A35:AH35">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
@@ -9881,151 +10151,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:XFD37 A40:XFD43">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A4:XFD4">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6:XFD6">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A7:XFD7">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A8:XFD8">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A9:XFD9">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A10:XFD10">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A24:XFD24 M26">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A34:XFD34">
-    <cfRule type="colorScale" priority="25">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A35:XFD35">
-    <cfRule type="colorScale" priority="22">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A38:XFD38">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A39:XFD39">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+  <conditionalFormatting sqref="AM39 AL38">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -10037,8 +10163,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="45">
+  <conditionalFormatting sqref="AO40:AP40 AP41 O14:AK14 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 O19:R19 T21 T22:U22 T23:V23 T24:W24 Z27 Z28:AA28 Z29:AB29 Z30:AC30 Z31:AD31 Z32:AE32 Z33:AF33 Z34:AG34 Z35:AH35 Z36:AI36 Z37:AJ37 Z40:AM40 Z41:AN41 Z42:AO42 Z43:AP43 G8:G12 T25:X25 O20:S25 F2:L3 E4:F4 AQ14:AQ32 H7:K7 L7:L11 G4:L6 AM24:AP28 P15:AK15 Q16:AK16 R17:AK17 S18:AK18 T19:AK19 U20:AK20 V21:AK21 W22:AK22 X23:AK23 Y24:AL24 Z25:AL25 AA26:AL26 AB27:AL27 AC28:AL28 AD29:AP29 AE30:AP30 AF31:AP31 AG32:AP32 AQ34:AQ37 AH33:AQ33 AI34:AP34 AJ35:AP35 AK36:AP36 AL37:AP37 AQ40:AQ42 N13:AK13 M2:AQ12 AN13:AQ13 AN14:AP23 AL13:AM23 M15:N25 M14 H11:J11 H12:K12 H35:Y37 L24:L25 H24:K34 G24:G37 G13:L23 F7:F16 D6:E16 D17:F37 D5 B4:C37 L26:Y34 B40:Y43">
+    <cfRule type="colorScale" priority="220">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10049,20 +10175,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="33">
+  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 D46:E46 B46 C45:E45 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 F45:M46 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N45:AQ56 AL57:AP67 O69:Y70 K60:N70">
+    <cfRule type="colorScale" priority="35">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10073,8 +10187,52 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2 B26:Y26">
-    <cfRule type="colorScale" priority="26">
+  <conditionalFormatting sqref="AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 X24 W23 V22 U21 T20 S19 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2">
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="49">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
+    <cfRule type="colorScale" priority="36">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="37">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR43:XFD43 A43:AP43 AQ42:XFD42 A42:AO42 AP41:XFD41 A41:AN41 AO40:XFD40 A40:AM40 AL37:XFD37 A37:AJ37 AK36:XFD36 A36:AI36 AJ35:XFD35 A35:AH35 AI34:XFD34 A34:AG34 AH33:XFD33 A33:AF33 AG32:XFD32 A32:AE32 AF31:XFD31 A31:AD31 AE30:XFD30 A30:AC30 AD29:XFD29 A29:AB29 AC28:XFD28 A28:AA28 AB27:XFD27 A27:Z27 AA26:XFD26 Z25:XFD25 A25:X25 Y24:XFD24 A24:W24 X23:XFD23 A23:V23 W22:XFD22 A22:U22 V21:XFD21 A21:T21 U20:XFD20 A20:S20 T19:XFD19 A19:R19 S18:XFD18 A18:Q18 R17:XFD17 A17:P17 Q16:XFD16 A16:O16 P15:XFD15 A15:N15 O14:XFD14 A14:M14 N13:XFD13 A13:L13 M12:XFD12 A12:K12 L11:XFD11 A11:J11 K10:XFD10 A10:I10 J9:XFD9 A9:H9 I8:XFD8 A8:G8 H7:XFD7 A7:F7 G6:XFD6 A6:E6 F5:XFD5 A5:D5 E4:XFD4 A4:C4 D3:XFD3 A3:B3 C2:XFD2 A2 A26:Y26">
+    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10085,67 +10243,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AQ37 B40:AQ43">
-    <cfRule type="colorScale" priority="28">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B7:AQ7">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I8:XFD8 A8:G8 G6:XFD6 A6:E6 E4:XFD4 A4:C4 C2:XFD2 A2 J9:XFD9 A9:H9 K10:XFD10 A10:I10 N13:XFD13 A13:L13 W22:XFD22 A22:U22 Y24:XFD24 A24:W24 AI34:XFD34 A34:AG34 AJ35:XFD35 A35:AH35">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
+  <conditionalFormatting sqref="AM39">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -10157,8 +10255,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AO40:AP40 AP41 O14:AK14 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 O19:R19 T21 T22:U22 T23:V23 T24:W24 Z27 Z28:AA28 Z29:AB29 Z30:AC30 Z31:AD31 Z32:AE32 Z33:AF33 Z34:AG34 Z35:AH35 Z36:AI36 Z37:AJ37 Z40:AM40 Z41:AN41 Z42:AO42 Z43:AP43 G8:G12 T25:X25 O20:S25 F2:L3 E4:F4 AQ14:AQ32 H7:K7 L7:L11 G4:L6 AM24:AP28 P15:AK15 Q16:AK16 R17:AK17 S18:AK18 T19:AK19 U20:AK20 V21:AK21 W22:AK22 X23:AK23 Y24:AL24 Z25:AL25 AA26:AL26 AB27:AL27 AC28:AL28 AD29:AP29 AE30:AP30 AF31:AP31 AG32:AP32 AQ34:AQ37 AH33:AQ33 AI34:AP34 AJ35:AP35 AK36:AP36 AL37:AP37 AQ40:AQ42 N13:AK13 M2:AQ12 AN13:AQ13 AN14:AP23 AL13:AM23 M15:N25 M14 H11:J11 H12:K12 H35:Y37 L24:L25 H24:K34 G24:G37 G13:L23 F7:F16 D6:E16 D17:F37 D5 B4:C37 L26:Y34 B40:Y43">
-    <cfRule type="colorScale" priority="215">
+  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 B2:AQ2">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10169,64 +10267,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 D46:E46 B46 C45:E45 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 F45:M46 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N45:AQ56 AL57:AP67 O69:Y70 K60:N70">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 X24 W23 V22 U21 T20 S19 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2">
-    <cfRule type="colorScale" priority="43">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="44">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="32">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AR43:XFD43 A43:AP43 AQ42:XFD42 A42:AO42 AP41:XFD41 A41:AN41 AO40:XFD40 A40:AM40 AL37:XFD37 A37:AJ37 AK36:XFD36 A36:AI36 AJ35:XFD35 A35:AH35 AI34:XFD34 A34:AG34 AH33:XFD33 A33:AF33 AG32:XFD32 A32:AE32 AF31:XFD31 A31:AD31 AE30:XFD30 A30:AC30 AD29:XFD29 A29:AB29 AC28:XFD28 A28:AA28 AB27:XFD27 A27:Z27 AA26:XFD26 Z25:XFD25 A25:X25 Y24:XFD24 A24:W24 X23:XFD23 A23:V23 W22:XFD22 A22:U22 V21:XFD21 A21:T21 U20:XFD20 A20:S20 T19:XFD19 A19:R19 S18:XFD18 A18:Q18 R17:XFD17 A17:P17 Q16:XFD16 A16:O16 P15:XFD15 A15:N15 O14:XFD14 A14:M14 N13:XFD13 A13:L13 M12:XFD12 A12:K12 L11:XFD11 A11:J11 K10:XFD10 A10:I10 J9:XFD9 A9:H9 I8:XFD8 A8:G8 H7:XFD7 A7:F7 G6:XFD6 A6:E6 F5:XFD5 A5:D5 E4:XFD4 A4:C4 D3:XFD3 A3:B3 C2:XFD2 A2 A26:Y26">
-    <cfRule type="colorScale" priority="10">
+  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -11026,7 +11068,7 @@
       </c>
       <c r="D36" s="24">
         <f>'Influence Matrix'!B37</f>
-        <v>-0.38</v>
+        <v>-0.17</v>
       </c>
       <c r="E36" t="s">
         <v>78</v>
@@ -11050,7 +11092,7 @@
       </c>
       <c r="D37" s="33">
         <f>'Influence Matrix'!B38</f>
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="G37" t="s">
         <v>72</v>
@@ -12057,7 +12099,7 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>29</v>
+        <v>173</v>
       </c>
       <c r="B36" s="1"/>
       <c r="C36" s="26"/>
@@ -12155,7 +12197,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F668546-2881-4668-A5C4-17806EA307E1}">
-  <dimension ref="B2:K17"/>
+  <dimension ref="B2:K20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -12327,12 +12369,22 @@
         <v>177</v>
       </c>
     </row>
-    <row r="17" spans="10:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="9:11" x14ac:dyDescent="0.25">
       <c r="J17" s="49" t="s">
         <v>174</v>
       </c>
       <c r="K17" s="49" t="s">
         <v>176</v>
+      </c>
+    </row>
+    <row r="19" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I19" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="20" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I20" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finished section for : Anatomy of the 42: Addiction
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="586" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24DF861D-60B6-4391-8939-3299BC1E975D}"/>
+  <xr:revisionPtr revIDLastSave="589" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97FDC044-1E79-478C-8F41-231CE9C1C556}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="194">
   <si>
     <t>Agriculture</t>
   </si>
@@ -648,6 +648,9 @@
   </si>
   <si>
     <t>Happiness</t>
+  </si>
+  <si>
+    <t>Welfare</t>
   </si>
 </sst>
 </file>
@@ -1996,7 +1999,7 @@
         <v>Transportation</v>
       </c>
       <c r="AQ1" s="21" t="str">
-        <v>Welfare Support</v>
+        <v>Welfare</v>
       </c>
       <c r="AR1" s="1"/>
       <c r="AS1" s="1"/>
@@ -7270,7 +7273,7 @@
         <v>Spirituality/God</v>
       </c>
       <c r="B39" s="13">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="C39" s="12">
         <v>0.27</v>
@@ -7835,10 +7838,10 @@
     <row r="43" spans="1:53" ht="17.100000000000001" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A43" s="45" t="str">
         <f>Sliders!A42</f>
-        <v>Welfare Support</v>
+        <v>Welfare</v>
       </c>
       <c r="B43" s="13">
-        <v>0.22</v>
+        <v>0.16</v>
       </c>
       <c r="C43" s="13">
         <v>0.18</v>
@@ -11113,7 +11116,7 @@
       </c>
       <c r="D38" s="24">
         <f>'Influence Matrix'!B39</f>
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="G38" t="s">
         <v>72</v>
@@ -11197,7 +11200,7 @@
       </c>
       <c r="D42" s="24">
         <f>'Influence Matrix'!B43</f>
-        <v>0.22</v>
+        <v>0.16</v>
       </c>
       <c r="G42" t="s">
         <v>72</v>
@@ -12171,7 +12174,7 @@
     </row>
     <row r="42" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
-        <v>44</v>
+        <v>193</v>
       </c>
       <c r="B42" s="1"/>
     </row>

</xml_diff>

<commit_message>
updated Anatomy of the 42, ver3.2.5
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="589" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97FDC044-1E79-478C-8F41-231CE9C1C556}"/>
+  <xr:revisionPtr revIDLastSave="591" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F20F3BE9-C922-4500-A5F6-3FEB9FC1A52B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -26,7 +26,6 @@
   <customWorkbookViews>
     <customWorkbookView name="ALL" guid="{C6883EF1-A235-4F7F-9B70-0CC3974E9739}" maximized="1" xWindow="1912" yWindow="126" windowWidth="1376" windowHeight="736" activeSheetId="1"/>
   </customWorkbookViews>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2306,7 +2305,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="13">
-        <v>0.14000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="D4" s="17">
         <v>1</v>
@@ -10034,7 +10033,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -10046,7 +10045,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
     <cfRule type="colorScale" priority="50">
       <colorScale>
         <cfvo type="min"/>
@@ -10070,7 +10069,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
     <cfRule type="colorScale" priority="38">
       <colorScale>
         <cfvo type="min"/>
@@ -10084,6 +10083,30 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2 B26:Y26">
     <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 B2:AQ2">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10118,7 +10141,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
     <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
@@ -10154,8 +10177,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM39 AL38">
+  <conditionalFormatting sqref="AL38 AM39">
     <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10246,42 +10281,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM39">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 B2:AQ2">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="90" orientation="portrait" horizontalDpi="4294967293" r:id="rId2"/>
 </worksheet>
@@ -11236,7 +11235,7 @@
       </c>
       <c r="D44" s="33">
         <f>'Influence Matrix'!C4</f>
-        <v>0.14000000000000001</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added research references to  directory
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="591" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F20F3BE9-C922-4500-A5F6-3FEB9FC1A52B}"/>
+  <xr:revisionPtr revIDLastSave="592" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{186256F3-249A-4775-89EA-DC408DF6ADC3}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -2447,7 +2447,7 @@
         <v>-0.16</v>
       </c>
       <c r="C5" s="12">
-        <v>0.13</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D5" s="13">
         <v>0</v>
@@ -11250,7 +11250,7 @@
       </c>
       <c r="D45" s="33">
         <f>'Influence Matrix'!C5</f>
-        <v>0.13</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added research reference to agr_cri; added edge summaries to Agriculture table in Anatomy of the 42
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="592" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{186256F3-249A-4775-89EA-DC408DF6ADC3}"/>
+  <xr:revisionPtr revIDLastSave="594" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6757CC74-BA46-4941-9B2A-96232E9B8EE2}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -2731,7 +2731,7 @@
         <v>0.15</v>
       </c>
       <c r="C7" s="12">
-        <v>-0.16</v>
+        <v>-0.12</v>
       </c>
       <c r="D7" s="13">
         <v>0</v>
@@ -2873,7 +2873,7 @@
         <v>0.3</v>
       </c>
       <c r="C8" s="12">
-        <v>-0.13</v>
+        <v>-0.14000000000000001</v>
       </c>
       <c r="D8" s="13">
         <v>-7.0000000000000007E-2</v>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="D47" s="33">
         <f>'Influence Matrix'!C7</f>
-        <v>-0.16</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="D48" s="33">
         <f>'Influence Matrix'!C8</f>
-        <v>-0.13</v>
+        <v>-0.14000000000000001</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added Agriculture resources to edges in repo and reflected in Anatomy of the 42 v3.2.6
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="594" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6757CC74-BA46-4941-9B2A-96232E9B8EE2}"/>
+  <xr:revisionPtr revIDLastSave="604" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{027DE954-337D-4663-9DE9-B7471FF1DEA5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="195">
   <si>
     <t>Agriculture</t>
   </si>
@@ -650,6 +650,9 @@
   </si>
   <si>
     <t>Welfare</t>
+  </si>
+  <si>
+    <t>Death Rate</t>
   </si>
 </sst>
 </file>
@@ -1896,7 +1899,7 @@
         <v>Crime</v>
       </c>
       <c r="I1" s="19" t="str">
-        <v>Deathrate</v>
+        <v>Death Rate</v>
       </c>
       <c r="J1" s="19" t="str">
         <v>Discrimination</v>
@@ -3009,13 +3012,13 @@
     <row r="9" spans="1:54" ht="17.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="str">
         <f>Sliders!A8</f>
-        <v>Deathrate</v>
+        <v>Death Rate</v>
       </c>
       <c r="B9" s="13">
         <v>0.31</v>
       </c>
       <c r="C9" s="12">
-        <v>0.14000000000000001</v>
+        <v>-0.17</v>
       </c>
       <c r="D9" s="13">
         <v>-0.13</v>
@@ -3157,7 +3160,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="14">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="D10" s="13">
         <v>0.27</v>
@@ -3299,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="C11" s="12">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="D11" s="13">
         <v>-0.2</v>
@@ -3441,7 +3444,7 @@
         <v>-7.0000000000000007E-2</v>
       </c>
       <c r="C12" s="12">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="D12" s="13">
         <v>0</v>
@@ -3583,7 +3586,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="12">
-        <v>-0.08</v>
+        <v>0</v>
       </c>
       <c r="D13" s="13">
         <v>0</v>
@@ -3725,7 +3728,7 @@
         <v>-0.17</v>
       </c>
       <c r="C14" s="12">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="D14" s="13">
         <v>-0.17</v>
@@ -3867,7 +3870,7 @@
         <v>-0.23</v>
       </c>
       <c r="C15" s="12">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
       <c r="D15" s="13">
         <v>-0.12</v>
@@ -10033,30 +10036,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="50">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B2">
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -10066,18 +10045,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10141,7 +10108,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
+  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
     <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
@@ -10177,7 +10156,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
+  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="38">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39 AL38">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -11310,7 +11313,7 @@
       </c>
       <c r="D49" s="33">
         <f>'Influence Matrix'!C9</f>
-        <v>0.14000000000000001</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -11325,7 +11328,7 @@
       </c>
       <c r="D50" s="33">
         <f>'Influence Matrix'!C10</f>
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -11340,7 +11343,7 @@
       </c>
       <c r="D51" s="33">
         <f>'Influence Matrix'!C11</f>
-        <v>0.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -11355,7 +11358,7 @@
       </c>
       <c r="D52" s="33">
         <f>'Influence Matrix'!C12</f>
-        <v>0.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -11370,7 +11373,7 @@
       </c>
       <c r="D53" s="33">
         <f>'Influence Matrix'!C13</f>
-        <v>-0.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -11385,7 +11388,7 @@
       </c>
       <c r="D54" s="33">
         <f>'Influence Matrix'!C14</f>
-        <v>0.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -11400,7 +11403,7 @@
       </c>
       <c r="D55" s="33">
         <f>'Influence Matrix'!C15</f>
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -11933,7 +11936,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>4</v>
+        <v>194</v>
       </c>
       <c r="B8" s="1"/>
     </row>

</xml_diff>

<commit_message>
Revised and updated Agriculture edgse for: Anatomy of the 42(v3.2.7)
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="604" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{027DE954-337D-4663-9DE9-B7471FF1DEA5}"/>
+  <xr:revisionPtr revIDLastSave="607" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F0C6DB6-AFEE-4575-9F7C-91E71CC5CFAE}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -4012,7 +4012,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="12">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
       <c r="D16" s="13">
         <v>0.1</v>
@@ -11418,7 +11418,7 @@
       </c>
       <c r="D56" s="33">
         <f>'Influence Matrix'!C16</f>
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Agriculture to Family Orientation updated
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="607" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F0C6DB6-AFEE-4575-9F7C-91E71CC5CFAE}"/>
+  <xr:revisionPtr revIDLastSave="608" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE836A99-FFC6-4E9A-9EAE-5EF768E7D12C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -4296,7 +4296,7 @@
         <v>-0.21</v>
       </c>
       <c r="C18" s="12">
-        <v>0.22</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="D18" s="13">
         <v>0.28999999999999998</v>
@@ -10036,6 +10036,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2">
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -10045,6 +10069,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="38">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10108,19 +10144,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
     <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
@@ -10156,31 +10180,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="50">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM39 AL38">
+  <conditionalFormatting sqref="AL38 AM39">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -11448,7 +11448,7 @@
       </c>
       <c r="D58" s="33">
         <f>'Influence Matrix'!C18</f>
-        <v>0.22</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Changed Gun Rights to Fireamrs in Influence Matrix spreadsheet
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="608" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE836A99-FFC6-4E9A-9EAE-5EF768E7D12C}"/>
+  <xr:revisionPtr revIDLastSave="683" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEA60180-11B0-4CD0-B55C-A8983EBB7449}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="196">
   <si>
     <t>Agriculture</t>
   </si>
@@ -653,6 +653,9 @@
   </si>
   <si>
     <t>Death Rate</t>
+  </si>
+  <si>
+    <t>Firearms</t>
   </si>
 </sst>
 </file>
@@ -1827,52 +1830,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{557F39C8-B3C6-46D2-B123-D33FD2398F37}">
   <dimension ref="A1:BB86"/>
-  <sheetFormatPr defaultColWidth="11.140625" defaultRowHeight="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" customWidth="1"/>
-    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" customWidth="1"/>
-    <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.140625" customWidth="1"/>
-    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16" customWidth="1"/>
-    <col min="17" max="17" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.85546875" customWidth="1"/>
-    <col min="20" max="20" width="10.7109375" customWidth="1"/>
-    <col min="21" max="21" width="11.140625" customWidth="1"/>
-    <col min="22" max="22" width="8.85546875" customWidth="1"/>
-    <col min="23" max="23" width="10.28515625" customWidth="1"/>
-    <col min="24" max="24" width="13.42578125" customWidth="1"/>
-    <col min="25" max="25" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14" customWidth="1"/>
-    <col min="29" max="29" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.140625" customWidth="1"/>
-    <col min="32" max="32" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="13.5703125" customWidth="1"/>
-    <col min="34" max="34" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11" customWidth="1"/>
-    <col min="37" max="37" width="15.85546875" customWidth="1"/>
-    <col min="38" max="38" width="15.5703125" customWidth="1"/>
-    <col min="39" max="39" width="13.42578125" customWidth="1"/>
-    <col min="40" max="40" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.5703125" customWidth="1"/>
-    <col min="43" max="43" width="13.85546875" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:54" s="23" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5"/>
@@ -1929,10 +1887,10 @@
         <v>Family Orientation</v>
       </c>
       <c r="S1" s="19" t="str">
+        <v>Firearms</v>
+      </c>
+      <c r="T1" s="19" t="str">
         <v>Freedom of Speech</v>
-      </c>
-      <c r="T1" s="19" t="str">
-        <v>Gun Rights</v>
       </c>
       <c r="U1" s="19" t="str">
         <v>HC Access</v>
@@ -2640,10 +2598,10 @@
         <v>-0.09</v>
       </c>
       <c r="S6" s="13">
+        <v>0</v>
+      </c>
+      <c r="T6" s="13">
         <v>-0.3</v>
-      </c>
-      <c r="T6" s="13">
-        <v>0</v>
       </c>
       <c r="U6" s="17">
         <v>0</v>
@@ -2924,10 +2882,10 @@
         <v>-0.26</v>
       </c>
       <c r="S8" s="13">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="T8" s="13">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="U8" s="17">
         <v>0</v>
@@ -3066,10 +3024,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="13">
-        <v>0</v>
+        <v>0.16</v>
       </c>
       <c r="T9" s="13">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="U9" s="17">
         <v>0</v>
@@ -3208,10 +3166,10 @@
         <v>0</v>
       </c>
       <c r="S10" s="13">
+        <v>0</v>
+      </c>
+      <c r="T10" s="13">
         <v>0.08</v>
-      </c>
-      <c r="T10" s="13">
-        <v>0</v>
       </c>
       <c r="U10" s="17">
         <v>0</v>
@@ -3492,10 +3450,10 @@
         <v>0</v>
       </c>
       <c r="S12" s="13">
+        <v>0</v>
+      </c>
+      <c r="T12" s="13">
         <v>0.02</v>
-      </c>
-      <c r="T12" s="13">
-        <v>0</v>
       </c>
       <c r="U12" s="17">
         <v>0</v>
@@ -3776,10 +3734,10 @@
         <v>0.02</v>
       </c>
       <c r="S14" s="13">
+        <v>0</v>
+      </c>
+      <c r="T14" s="13">
         <v>0.05</v>
-      </c>
-      <c r="T14" s="13">
-        <v>0</v>
       </c>
       <c r="U14" s="17">
         <v>0</v>
@@ -3918,10 +3876,10 @@
         <v>0.02</v>
       </c>
       <c r="S15" s="13">
+        <v>0</v>
+      </c>
+      <c r="T15" s="13">
         <v>0.03</v>
-      </c>
-      <c r="T15" s="13">
-        <v>0</v>
       </c>
       <c r="U15" s="17">
         <v>0</v>
@@ -4202,10 +4160,10 @@
         <v>0</v>
       </c>
       <c r="S17" s="13">
+        <v>0</v>
+      </c>
+      <c r="T17" s="13">
         <v>0.03</v>
-      </c>
-      <c r="T17" s="13">
-        <v>0</v>
       </c>
       <c r="U17" s="17">
         <v>0</v>
@@ -4344,10 +4302,10 @@
         <v>1</v>
       </c>
       <c r="S18" s="13">
+        <v>0</v>
+      </c>
+      <c r="T18" s="13">
         <v>0.05</v>
-      </c>
-      <c r="T18" s="13">
-        <v>0</v>
       </c>
       <c r="U18" s="17">
         <v>0</v>
@@ -4432,46 +4390,46 @@
     <row r="19" spans="1:53" ht="17.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="str">
         <f>Sliders!A18</f>
-        <v>Freedom of Speech</v>
+        <v>Firearms</v>
       </c>
       <c r="B19" s="13">
-        <v>0</v>
+        <v>-0.06</v>
       </c>
       <c r="C19" s="12">
-        <v>-0.08</v>
+        <v>0.01</v>
       </c>
       <c r="D19" s="13">
-        <v>-0.33</v>
+        <v>-0.14000000000000001</v>
       </c>
       <c r="E19" s="13">
         <v>0</v>
       </c>
       <c r="F19" s="13">
-        <v>-0.28000000000000003</v>
+        <v>0</v>
       </c>
       <c r="G19" s="13">
         <v>0</v>
       </c>
       <c r="H19" s="13">
-        <v>-0.04</v>
+        <v>-0.21</v>
       </c>
       <c r="I19" s="13">
         <v>0</v>
       </c>
       <c r="J19" s="13">
-        <v>-0.12</v>
+        <v>0</v>
       </c>
       <c r="K19" s="13">
         <v>0</v>
       </c>
       <c r="L19" s="13">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="M19" s="13">
         <v>0</v>
       </c>
       <c r="N19" s="13">
-        <v>0.09</v>
+        <v>0.03</v>
       </c>
       <c r="O19" s="13">
         <v>0</v>
@@ -4480,10 +4438,10 @@
         <v>0</v>
       </c>
       <c r="Q19" s="13">
-        <v>7.0000000000000007E-2</v>
+        <v>0.03</v>
       </c>
       <c r="R19" s="13">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="S19" s="17">
         <v>1</v>
@@ -4574,46 +4532,46 @@
     <row r="20" spans="1:53" ht="17.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="str">
         <f>Sliders!A19</f>
-        <v>Gun Rights</v>
+        <v>Freedom of Speech</v>
       </c>
       <c r="B20" s="13">
-        <v>-0.06</v>
+        <v>0</v>
       </c>
       <c r="C20" s="12">
-        <v>0.01</v>
+        <v>-0.08</v>
       </c>
       <c r="D20" s="13">
-        <v>-0.14000000000000001</v>
+        <v>-0.33</v>
       </c>
       <c r="E20" s="13">
         <v>0</v>
       </c>
       <c r="F20" s="13">
-        <v>0</v>
+        <v>-0.28000000000000003</v>
       </c>
       <c r="G20" s="13">
         <v>0</v>
       </c>
       <c r="H20" s="13">
-        <v>-0.21</v>
+        <v>-0.04</v>
       </c>
       <c r="I20" s="13">
         <v>0</v>
       </c>
       <c r="J20" s="13">
-        <v>0</v>
+        <v>-0.12</v>
       </c>
       <c r="K20" s="13">
         <v>0</v>
       </c>
       <c r="L20" s="13">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="M20" s="13">
         <v>0</v>
       </c>
       <c r="N20" s="13">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
       <c r="O20" s="13">
         <v>0</v>
@@ -4622,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="Q20" s="13">
-        <v>0.03</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="R20" s="13">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="S20" s="13">
         <v>0</v>
@@ -4779,7 +4737,7 @@
         <v>1</v>
       </c>
       <c r="V21" s="17">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="W21" s="17">
         <v>0</v>
@@ -5054,16 +5012,16 @@
         <v>0</v>
       </c>
       <c r="S23" s="13">
+        <v>0</v>
+      </c>
+      <c r="T23" s="13">
         <v>0.11</v>
       </c>
-      <c r="T23" s="13">
-        <v>0</v>
-      </c>
       <c r="U23" s="17">
         <v>0</v>
       </c>
       <c r="V23" s="17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W23" s="17">
         <v>1</v>
@@ -5622,10 +5580,10 @@
         <v>0.16</v>
       </c>
       <c r="S27" s="13">
+        <v>0</v>
+      </c>
+      <c r="T27" s="13">
         <v>0.27</v>
-      </c>
-      <c r="T27" s="13">
-        <v>0</v>
       </c>
       <c r="U27" s="17">
         <v>0</v>
@@ -5764,10 +5722,10 @@
         <v>0</v>
       </c>
       <c r="S28" s="13">
+        <v>-0.17</v>
+      </c>
+      <c r="T28" s="13">
         <v>0.12</v>
-      </c>
-      <c r="T28" s="13">
-        <v>-0.17</v>
       </c>
       <c r="U28" s="17">
         <v>0</v>
@@ -5906,10 +5864,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="S29" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="T29" s="13">
         <v>0.4</v>
-      </c>
-      <c r="T29" s="13">
-        <v>0.2</v>
       </c>
       <c r="U29" s="17">
         <v>0</v>
@@ -6048,10 +6006,10 @@
         <v>0</v>
       </c>
       <c r="S30" s="13">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="T30" s="13">
         <v>0.18</v>
-      </c>
-      <c r="T30" s="13">
-        <v>7.0000000000000007E-2</v>
       </c>
       <c r="U30" s="17">
         <v>0</v>
@@ -6190,10 +6148,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="S31" s="13">
+        <v>-0.09</v>
+      </c>
+      <c r="T31" s="13">
         <v>0.2</v>
-      </c>
-      <c r="T31" s="13">
-        <v>-0.09</v>
       </c>
       <c r="U31" s="17">
         <v>0</v>
@@ -6900,10 +6858,10 @@
         <v>0</v>
       </c>
       <c r="S36" s="13">
+        <v>-0.05</v>
+      </c>
+      <c r="T36" s="13">
         <v>0.09</v>
-      </c>
-      <c r="T36" s="13">
-        <v>-0.05</v>
       </c>
       <c r="U36" s="17">
         <v>0</v>
@@ -7987,25 +7945,6 @@
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
-      <c r="P45" s="2"/>
-      <c r="Q45" s="2"/>
-      <c r="R45" s="2"/>
-      <c r="S45" s="2"/>
-      <c r="T45" s="2"/>
-      <c r="U45" s="2"/>
-      <c r="V45" s="2"/>
-      <c r="W45" s="2"/>
-      <c r="X45" s="2"/>
-      <c r="Y45" s="2"/>
-      <c r="Z45" s="2"/>
       <c r="AA45" s="2"/>
       <c r="AB45" s="2"/>
       <c r="AC45" s="2"/>
@@ -9880,8 +9819,114 @@
       <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
     </customSheetView>
   </customSheetViews>
-  <conditionalFormatting sqref="A2:XFD2">
-    <cfRule type="colorScale" priority="18">
+  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7">
+    <cfRule type="colorScale" priority="37">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL38 AM39">
+    <cfRule type="colorScale" priority="40">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39">
+    <cfRule type="colorScale" priority="35">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 B46 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 D46:M46 C45:G45 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N46:AQ56 AA45:AQ45 AL57:AP67 O69:Y70 K60:N70">
+    <cfRule type="colorScale" priority="66">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 V22 U21 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2 W23">
+    <cfRule type="colorScale" priority="79">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="80">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9892,7 +9937,197 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:XFD37 A40:XFD43">
+  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
+    <cfRule type="colorScale" priority="67">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="68">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T19 S20">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B1048576">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:C1048576 C2">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D5:D1048576 D2:D3">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6:E1048576 E2:E4">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7:F1048576 F2:F5">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8:G1048576 G2:G6">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9:H1048576 H2:H7">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I10:I1048576 I2:I8">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J11:J1048576 J2:J9">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12:K1048576 K2:K10">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L13:L1048576 L2:L11">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M14:M1048576 M2:M12">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
@@ -9904,8 +10139,200 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:XFD4">
-    <cfRule type="colorScale" priority="20">
+  <conditionalFormatting sqref="N15:N1048576 N2:N13">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O16:O1048576 O2:O14">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P17:P1048576 P2:P15">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q18:Q1048576 Q2:Q16">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R19:R1048576 R2:R17">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2:T18 S44:S1048576 T20:T43">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S19 T44:T1048576 S21:S43">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U22:U1048576 U2:U20">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V44:V1048576">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T21:T25 T19 U19:U20 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 B19:R37 S20:S37 X24 U22:U25 T26:U37 B40:U43">
+    <cfRule type="colorScale" priority="357">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="474">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="597">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T21:T25 B19:R19 O14:R14 S14:S18 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 G8:G12 F2:L3 E4:F4 H7:K7 L7:L11 G4:L6 P15:R15 Q16:R16 R17 T14:T19 U14:U20 N13:U13 M2:U12 M15:N18 M20:R25 M14 H11:J11 H12:K12 H35:R37 S20:S37 L24:L25 H24:K34 G24:G37 G13:L18 G20:L23 F7:F16 D6:E16 D17:F18 D5 B4:C18 B20:F37 L26:R34 X24 U22:U25 T26:U37 B40:U43">
+    <cfRule type="colorScale" priority="768">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR40:XFD43 T21:T25 U20 T2:U19 S2:S18 A18:Q18 R17 A17:P17 Q16:R16 A16:O16 P15:R15 A15:N15 O14:R14 A14:M14 N13:R13 A13:L13 M12:R12 A12:K12 L11:R11 A11:J11 K10:R10 A10:I10 J9:R9 A9:H9 I8:R8 A8:G8 H7:R7 A7:F7 G6:R6 A6:E6 F5:R5 A5:D5 E4:R4 A4:C4 D3:R3 A3:B3 C2:R2 A2 A19:R37 S20:S37 X24 AR2:XFD37 U22:U25 T26:U37 A40:U43">
+    <cfRule type="colorScale" priority="950">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S21:S43 T20:T43 U19:U20 B19:R43 T2:U18 S2:S19 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="1070">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:U2 AR2:XFD2">
+    <cfRule type="colorScale" priority="1071">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9916,8 +10343,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A6:XFD6">
-    <cfRule type="colorScale" priority="21">
+  <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
+    <cfRule type="colorScale" priority="1074">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:U4 AR4:XFD4">
+    <cfRule type="colorScale" priority="1080">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9928,8 +10367,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:XFD7">
-    <cfRule type="colorScale" priority="22">
+  <conditionalFormatting sqref="A6:U6 AR6:XFD6">
+    <cfRule type="colorScale" priority="1083">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9940,8 +10379,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A8:XFD8">
-    <cfRule type="colorScale" priority="23">
+  <conditionalFormatting sqref="A7:U7 AR7:XFD7">
+    <cfRule type="colorScale" priority="1086">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9952,8 +10391,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A9:XFD9">
-    <cfRule type="colorScale" priority="24">
+  <conditionalFormatting sqref="A8:U8 AR8:XFD8">
+    <cfRule type="colorScale" priority="1089">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9964,8 +10403,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A10:XFD10">
-    <cfRule type="colorScale" priority="25">
+  <conditionalFormatting sqref="A9:U9 AR9:XFD9">
+    <cfRule type="colorScale" priority="1092">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9976,8 +10415,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A24:XFD24 M26">
-    <cfRule type="colorScale" priority="26">
+  <conditionalFormatting sqref="A10:U10 AR10:XFD10">
+    <cfRule type="colorScale" priority="1095">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9988,8 +10427,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A34:XFD34">
-    <cfRule type="colorScale" priority="30">
+  <conditionalFormatting sqref="A24:U24 M26 X24 AR24:XFD24">
+    <cfRule type="colorScale" priority="1098">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10000,8 +10439,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A35:XFD35">
-    <cfRule type="colorScale" priority="27">
+  <conditionalFormatting sqref="A34:U34 AH34 AR34:XFD34">
+    <cfRule type="colorScale" priority="1102">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10012,8 +10451,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A38:XFD38">
-    <cfRule type="colorScale" priority="12">
+  <conditionalFormatting sqref="A35:U35 AI35 AR35:XFD35">
+    <cfRule type="colorScale" priority="1105">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10024,7 +10463,67 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A39:XFD39">
+  <conditionalFormatting sqref="A38:U38 AL38 AR38:XFD38">
+    <cfRule type="colorScale" priority="1108">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A39:U39 AM39 AR39:XFD39">
+    <cfRule type="colorScale" priority="1111">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7:U7">
+    <cfRule type="colorScale" priority="1196">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I8:R8 A8:G8 A6:E6 A4:C4 A2 J9:R9 A9:H9 K10:R10 A10:I10 A13:L13 A22:U22 AR34:XFD35 S8:U10 G6:U6 E4:U4 C2:U2 N13:U13 AR22:XFD22 A24:U24 AR13:XFD13 AR2:XFD2 AR4:XFD4 AR6:XFD6 AR8:XFD10 X24 AR24:XFD24 A34:U35">
+    <cfRule type="colorScale" priority="1199">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X24">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -10036,20 +10535,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="50">
+  <conditionalFormatting sqref="X24">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10060,7 +10547,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2">
+  <conditionalFormatting sqref="T21:T1048576 T2:T19">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S20:S1048576 S2:S18">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19 T20 X24">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -10072,208 +10583,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2 B26:Y26">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 B2:AQ2">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2">
+  <conditionalFormatting sqref="X44:X1048576">
     <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AQ37 B40:AQ43">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B7:AQ7">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I8:XFD8 A8:G8 G6:XFD6 A6:E6 E4:XFD4 A4:C4 C2:XFD2 A2 J9:XFD9 A9:H9 K10:XFD10 A10:I10 N13:XFD13 A13:L13 W22:XFD22 A22:U22 Y24:XFD24 A24:W24 AI34:XFD34 A34:AG34 AJ35:XFD35 A35:AH35">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM39">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO40:AP40 AP41 O14:AK14 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 O19:R19 T21 T22:U22 T23:V23 T24:W24 Z27 Z28:AA28 Z29:AB29 Z30:AC30 Z31:AD31 Z32:AE32 Z33:AF33 Z34:AG34 Z35:AH35 Z36:AI36 Z37:AJ37 Z40:AM40 Z41:AN41 Z42:AO42 Z43:AP43 G8:G12 T25:X25 O20:S25 F2:L3 E4:F4 AQ14:AQ32 H7:K7 L7:L11 G4:L6 AM24:AP28 P15:AK15 Q16:AK16 R17:AK17 S18:AK18 T19:AK19 U20:AK20 V21:AK21 W22:AK22 X23:AK23 Y24:AL24 Z25:AL25 AA26:AL26 AB27:AL27 AC28:AL28 AD29:AP29 AE30:AP30 AF31:AP31 AG32:AP32 AQ34:AQ37 AH33:AQ33 AI34:AP34 AJ35:AP35 AK36:AP36 AL37:AP37 AQ40:AQ42 N13:AK13 M2:AQ12 AN13:AQ13 AN14:AP23 AL13:AM23 M15:N25 M14 H11:J11 H12:K12 H35:Y37 L24:L25 H24:K34 G24:G37 G13:L23 F7:F16 D6:E16 D17:F37 D5 B4:C37 L26:Y34 B40:Y43">
-    <cfRule type="colorScale" priority="220">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 D46:E46 B46 C45:E45 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 F45:M46 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N45:AQ56 AL57:AP67 O69:Y70 K60:N70">
-    <cfRule type="colorScale" priority="35">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 X24 W23 V22 U21 T20 S19 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2">
-    <cfRule type="colorScale" priority="48">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="49">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
-    <cfRule type="colorScale" priority="36">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="37">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AR43:XFD43 A43:AP43 AQ42:XFD42 A42:AO42 AP41:XFD41 A41:AN41 AO40:XFD40 A40:AM40 AL37:XFD37 A37:AJ37 AK36:XFD36 A36:AI36 AJ35:XFD35 A35:AH35 AI34:XFD34 A34:AG34 AH33:XFD33 A33:AF33 AG32:XFD32 A32:AE32 AF31:XFD31 A31:AD31 AE30:XFD30 A30:AC30 AD29:XFD29 A29:AB29 AC28:XFD28 A28:AA28 AB27:XFD27 A27:Z27 AA26:XFD26 Z25:XFD25 A25:X25 Y24:XFD24 A24:W24 X23:XFD23 A23:V23 W22:XFD22 A22:U22 V21:XFD21 A21:T21 U20:XFD20 A20:S20 T19:XFD19 A19:R19 S18:XFD18 A18:Q18 R17:XFD17 A17:P17 Q16:XFD16 A16:O16 P15:XFD15 A15:N15 O14:XFD14 A14:M14 N13:XFD13 A13:L13 M12:XFD12 A12:K12 L11:XFD11 A11:J11 K10:XFD10 A10:I10 J9:XFD9 A9:H9 I8:XFD8 A8:G8 H7:XFD7 A7:F7 G6:XFD6 A6:E6 F5:XFD5 A5:D5 E4:XFD4 A4:C4 D3:XFD3 A3:B3 C2:XFD2 A2 A26:Y26">
-    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10694,7 +11005,7 @@
         <v>43</v>
       </c>
       <c r="D18" s="33">
-        <f>'Influence Matrix'!B19</f>
+        <f>'Influence Matrix'!B20</f>
         <v>0</v>
       </c>
       <c r="G18" t="s">
@@ -10715,7 +11026,7 @@
         <v>19</v>
       </c>
       <c r="D19" s="24">
-        <f>'Influence Matrix'!B20</f>
+        <f>'Influence Matrix'!B19</f>
         <v>-0.06</v>
       </c>
       <c r="G19" t="s">
@@ -11462,7 +11773,7 @@
         <v>43</v>
       </c>
       <c r="D59" s="33">
-        <f>'Influence Matrix'!C19</f>
+        <f>'Influence Matrix'!C20</f>
         <v>-0.08</v>
       </c>
     </row>
@@ -11477,7 +11788,7 @@
         <v>19</v>
       </c>
       <c r="D60" s="33">
-        <f>'Influence Matrix'!C20</f>
+        <f>'Influence Matrix'!C19</f>
         <v>0.01</v>
       </c>
     </row>
@@ -11996,13 +12307,13 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>43</v>
+        <v>195</v>
       </c>
       <c r="B18" s="1"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="B19" s="1"/>
     </row>

</xml_diff>

<commit_message>
Changed Gun Rights to Firearms
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="608" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE836A99-FFC6-4E9A-9EAE-5EF768E7D12C}"/>
+  <xr:revisionPtr revIDLastSave="683" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEA60180-11B0-4CD0-B55C-A8983EBB7449}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="196">
   <si>
     <t>Agriculture</t>
   </si>
@@ -653,6 +653,9 @@
   </si>
   <si>
     <t>Death Rate</t>
+  </si>
+  <si>
+    <t>Firearms</t>
   </si>
 </sst>
 </file>
@@ -1827,52 +1830,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{557F39C8-B3C6-46D2-B123-D33FD2398F37}">
   <dimension ref="A1:BB86"/>
-  <sheetFormatPr defaultColWidth="11.140625" defaultRowHeight="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" customWidth="1"/>
-    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" customWidth="1"/>
-    <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.140625" customWidth="1"/>
-    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16" customWidth="1"/>
-    <col min="17" max="17" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.85546875" customWidth="1"/>
-    <col min="20" max="20" width="10.7109375" customWidth="1"/>
-    <col min="21" max="21" width="11.140625" customWidth="1"/>
-    <col min="22" max="22" width="8.85546875" customWidth="1"/>
-    <col min="23" max="23" width="10.28515625" customWidth="1"/>
-    <col min="24" max="24" width="13.42578125" customWidth="1"/>
-    <col min="25" max="25" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14" customWidth="1"/>
-    <col min="29" max="29" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.140625" customWidth="1"/>
-    <col min="32" max="32" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="13.5703125" customWidth="1"/>
-    <col min="34" max="34" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11" customWidth="1"/>
-    <col min="37" max="37" width="15.85546875" customWidth="1"/>
-    <col min="38" max="38" width="15.5703125" customWidth="1"/>
-    <col min="39" max="39" width="13.42578125" customWidth="1"/>
-    <col min="40" max="40" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.5703125" customWidth="1"/>
-    <col min="43" max="43" width="13.85546875" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:54" s="23" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5"/>
@@ -1929,10 +1887,10 @@
         <v>Family Orientation</v>
       </c>
       <c r="S1" s="19" t="str">
+        <v>Firearms</v>
+      </c>
+      <c r="T1" s="19" t="str">
         <v>Freedom of Speech</v>
-      </c>
-      <c r="T1" s="19" t="str">
-        <v>Gun Rights</v>
       </c>
       <c r="U1" s="19" t="str">
         <v>HC Access</v>
@@ -2640,10 +2598,10 @@
         <v>-0.09</v>
       </c>
       <c r="S6" s="13">
+        <v>0</v>
+      </c>
+      <c r="T6" s="13">
         <v>-0.3</v>
-      </c>
-      <c r="T6" s="13">
-        <v>0</v>
       </c>
       <c r="U6" s="17">
         <v>0</v>
@@ -2924,10 +2882,10 @@
         <v>-0.26</v>
       </c>
       <c r="S8" s="13">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="T8" s="13">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="U8" s="17">
         <v>0</v>
@@ -3066,10 +3024,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="13">
-        <v>0</v>
+        <v>0.16</v>
       </c>
       <c r="T9" s="13">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="U9" s="17">
         <v>0</v>
@@ -3208,10 +3166,10 @@
         <v>0</v>
       </c>
       <c r="S10" s="13">
+        <v>0</v>
+      </c>
+      <c r="T10" s="13">
         <v>0.08</v>
-      </c>
-      <c r="T10" s="13">
-        <v>0</v>
       </c>
       <c r="U10" s="17">
         <v>0</v>
@@ -3492,10 +3450,10 @@
         <v>0</v>
       </c>
       <c r="S12" s="13">
+        <v>0</v>
+      </c>
+      <c r="T12" s="13">
         <v>0.02</v>
-      </c>
-      <c r="T12" s="13">
-        <v>0</v>
       </c>
       <c r="U12" s="17">
         <v>0</v>
@@ -3776,10 +3734,10 @@
         <v>0.02</v>
       </c>
       <c r="S14" s="13">
+        <v>0</v>
+      </c>
+      <c r="T14" s="13">
         <v>0.05</v>
-      </c>
-      <c r="T14" s="13">
-        <v>0</v>
       </c>
       <c r="U14" s="17">
         <v>0</v>
@@ -3918,10 +3876,10 @@
         <v>0.02</v>
       </c>
       <c r="S15" s="13">
+        <v>0</v>
+      </c>
+      <c r="T15" s="13">
         <v>0.03</v>
-      </c>
-      <c r="T15" s="13">
-        <v>0</v>
       </c>
       <c r="U15" s="17">
         <v>0</v>
@@ -4202,10 +4160,10 @@
         <v>0</v>
       </c>
       <c r="S17" s="13">
+        <v>0</v>
+      </c>
+      <c r="T17" s="13">
         <v>0.03</v>
-      </c>
-      <c r="T17" s="13">
-        <v>0</v>
       </c>
       <c r="U17" s="17">
         <v>0</v>
@@ -4344,10 +4302,10 @@
         <v>1</v>
       </c>
       <c r="S18" s="13">
+        <v>0</v>
+      </c>
+      <c r="T18" s="13">
         <v>0.05</v>
-      </c>
-      <c r="T18" s="13">
-        <v>0</v>
       </c>
       <c r="U18" s="17">
         <v>0</v>
@@ -4432,46 +4390,46 @@
     <row r="19" spans="1:53" ht="17.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="str">
         <f>Sliders!A18</f>
-        <v>Freedom of Speech</v>
+        <v>Firearms</v>
       </c>
       <c r="B19" s="13">
-        <v>0</v>
+        <v>-0.06</v>
       </c>
       <c r="C19" s="12">
-        <v>-0.08</v>
+        <v>0.01</v>
       </c>
       <c r="D19" s="13">
-        <v>-0.33</v>
+        <v>-0.14000000000000001</v>
       </c>
       <c r="E19" s="13">
         <v>0</v>
       </c>
       <c r="F19" s="13">
-        <v>-0.28000000000000003</v>
+        <v>0</v>
       </c>
       <c r="G19" s="13">
         <v>0</v>
       </c>
       <c r="H19" s="13">
-        <v>-0.04</v>
+        <v>-0.21</v>
       </c>
       <c r="I19" s="13">
         <v>0</v>
       </c>
       <c r="J19" s="13">
-        <v>-0.12</v>
+        <v>0</v>
       </c>
       <c r="K19" s="13">
         <v>0</v>
       </c>
       <c r="L19" s="13">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="M19" s="13">
         <v>0</v>
       </c>
       <c r="N19" s="13">
-        <v>0.09</v>
+        <v>0.03</v>
       </c>
       <c r="O19" s="13">
         <v>0</v>
@@ -4480,10 +4438,10 @@
         <v>0</v>
       </c>
       <c r="Q19" s="13">
-        <v>7.0000000000000007E-2</v>
+        <v>0.03</v>
       </c>
       <c r="R19" s="13">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="S19" s="17">
         <v>1</v>
@@ -4574,46 +4532,46 @@
     <row r="20" spans="1:53" ht="17.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="str">
         <f>Sliders!A19</f>
-        <v>Gun Rights</v>
+        <v>Freedom of Speech</v>
       </c>
       <c r="B20" s="13">
-        <v>-0.06</v>
+        <v>0</v>
       </c>
       <c r="C20" s="12">
-        <v>0.01</v>
+        <v>-0.08</v>
       </c>
       <c r="D20" s="13">
-        <v>-0.14000000000000001</v>
+        <v>-0.33</v>
       </c>
       <c r="E20" s="13">
         <v>0</v>
       </c>
       <c r="F20" s="13">
-        <v>0</v>
+        <v>-0.28000000000000003</v>
       </c>
       <c r="G20" s="13">
         <v>0</v>
       </c>
       <c r="H20" s="13">
-        <v>-0.21</v>
+        <v>-0.04</v>
       </c>
       <c r="I20" s="13">
         <v>0</v>
       </c>
       <c r="J20" s="13">
-        <v>0</v>
+        <v>-0.12</v>
       </c>
       <c r="K20" s="13">
         <v>0</v>
       </c>
       <c r="L20" s="13">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="M20" s="13">
         <v>0</v>
       </c>
       <c r="N20" s="13">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
       <c r="O20" s="13">
         <v>0</v>
@@ -4622,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="Q20" s="13">
-        <v>0.03</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="R20" s="13">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="S20" s="13">
         <v>0</v>
@@ -4779,7 +4737,7 @@
         <v>1</v>
       </c>
       <c r="V21" s="17">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="W21" s="17">
         <v>0</v>
@@ -5054,16 +5012,16 @@
         <v>0</v>
       </c>
       <c r="S23" s="13">
+        <v>0</v>
+      </c>
+      <c r="T23" s="13">
         <v>0.11</v>
       </c>
-      <c r="T23" s="13">
-        <v>0</v>
-      </c>
       <c r="U23" s="17">
         <v>0</v>
       </c>
       <c r="V23" s="17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W23" s="17">
         <v>1</v>
@@ -5622,10 +5580,10 @@
         <v>0.16</v>
       </c>
       <c r="S27" s="13">
+        <v>0</v>
+      </c>
+      <c r="T27" s="13">
         <v>0.27</v>
-      </c>
-      <c r="T27" s="13">
-        <v>0</v>
       </c>
       <c r="U27" s="17">
         <v>0</v>
@@ -5764,10 +5722,10 @@
         <v>0</v>
       </c>
       <c r="S28" s="13">
+        <v>-0.17</v>
+      </c>
+      <c r="T28" s="13">
         <v>0.12</v>
-      </c>
-      <c r="T28" s="13">
-        <v>-0.17</v>
       </c>
       <c r="U28" s="17">
         <v>0</v>
@@ -5906,10 +5864,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="S29" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="T29" s="13">
         <v>0.4</v>
-      </c>
-      <c r="T29" s="13">
-        <v>0.2</v>
       </c>
       <c r="U29" s="17">
         <v>0</v>
@@ -6048,10 +6006,10 @@
         <v>0</v>
       </c>
       <c r="S30" s="13">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="T30" s="13">
         <v>0.18</v>
-      </c>
-      <c r="T30" s="13">
-        <v>7.0000000000000007E-2</v>
       </c>
       <c r="U30" s="17">
         <v>0</v>
@@ -6190,10 +6148,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="S31" s="13">
+        <v>-0.09</v>
+      </c>
+      <c r="T31" s="13">
         <v>0.2</v>
-      </c>
-      <c r="T31" s="13">
-        <v>-0.09</v>
       </c>
       <c r="U31" s="17">
         <v>0</v>
@@ -6900,10 +6858,10 @@
         <v>0</v>
       </c>
       <c r="S36" s="13">
+        <v>-0.05</v>
+      </c>
+      <c r="T36" s="13">
         <v>0.09</v>
-      </c>
-      <c r="T36" s="13">
-        <v>-0.05</v>
       </c>
       <c r="U36" s="17">
         <v>0</v>
@@ -7987,25 +7945,6 @@
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
-      <c r="P45" s="2"/>
-      <c r="Q45" s="2"/>
-      <c r="R45" s="2"/>
-      <c r="S45" s="2"/>
-      <c r="T45" s="2"/>
-      <c r="U45" s="2"/>
-      <c r="V45" s="2"/>
-      <c r="W45" s="2"/>
-      <c r="X45" s="2"/>
-      <c r="Y45" s="2"/>
-      <c r="Z45" s="2"/>
       <c r="AA45" s="2"/>
       <c r="AB45" s="2"/>
       <c r="AC45" s="2"/>
@@ -9880,8 +9819,114 @@
       <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
     </customSheetView>
   </customSheetViews>
-  <conditionalFormatting sqref="A2:XFD2">
-    <cfRule type="colorScale" priority="18">
+  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7">
+    <cfRule type="colorScale" priority="37">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL38 AM39">
+    <cfRule type="colorScale" priority="40">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39">
+    <cfRule type="colorScale" priority="35">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 B46 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 D46:M46 C45:G45 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N46:AQ56 AA45:AQ45 AL57:AP67 O69:Y70 K60:N70">
+    <cfRule type="colorScale" priority="66">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 V22 U21 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2 W23">
+    <cfRule type="colorScale" priority="79">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="80">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9892,7 +9937,197 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:XFD37 A40:XFD43">
+  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
+    <cfRule type="colorScale" priority="67">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="68">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T19 S20">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B1048576">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:C1048576 C2">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D5:D1048576 D2:D3">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6:E1048576 E2:E4">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7:F1048576 F2:F5">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8:G1048576 G2:G6">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9:H1048576 H2:H7">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I10:I1048576 I2:I8">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J11:J1048576 J2:J9">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12:K1048576 K2:K10">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L13:L1048576 L2:L11">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M14:M1048576 M2:M12">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
@@ -9904,8 +10139,200 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:XFD4">
-    <cfRule type="colorScale" priority="20">
+  <conditionalFormatting sqref="N15:N1048576 N2:N13">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O16:O1048576 O2:O14">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P17:P1048576 P2:P15">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q18:Q1048576 Q2:Q16">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R19:R1048576 R2:R17">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2:T18 S44:S1048576 T20:T43">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S19 T44:T1048576 S21:S43">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U22:U1048576 U2:U20">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V44:V1048576">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T21:T25 T19 U19:U20 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 B19:R37 S20:S37 X24 U22:U25 T26:U37 B40:U43">
+    <cfRule type="colorScale" priority="357">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="474">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="597">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T21:T25 B19:R19 O14:R14 S14:S18 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 G8:G12 F2:L3 E4:F4 H7:K7 L7:L11 G4:L6 P15:R15 Q16:R16 R17 T14:T19 U14:U20 N13:U13 M2:U12 M15:N18 M20:R25 M14 H11:J11 H12:K12 H35:R37 S20:S37 L24:L25 H24:K34 G24:G37 G13:L18 G20:L23 F7:F16 D6:E16 D17:F18 D5 B4:C18 B20:F37 L26:R34 X24 U22:U25 T26:U37 B40:U43">
+    <cfRule type="colorScale" priority="768">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR40:XFD43 T21:T25 U20 T2:U19 S2:S18 A18:Q18 R17 A17:P17 Q16:R16 A16:O16 P15:R15 A15:N15 O14:R14 A14:M14 N13:R13 A13:L13 M12:R12 A12:K12 L11:R11 A11:J11 K10:R10 A10:I10 J9:R9 A9:H9 I8:R8 A8:G8 H7:R7 A7:F7 G6:R6 A6:E6 F5:R5 A5:D5 E4:R4 A4:C4 D3:R3 A3:B3 C2:R2 A2 A19:R37 S20:S37 X24 AR2:XFD37 U22:U25 T26:U37 A40:U43">
+    <cfRule type="colorScale" priority="950">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S21:S43 T20:T43 U19:U20 B19:R43 T2:U18 S2:S19 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="1070">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:U2 AR2:XFD2">
+    <cfRule type="colorScale" priority="1071">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9916,8 +10343,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A6:XFD6">
-    <cfRule type="colorScale" priority="21">
+  <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
+    <cfRule type="colorScale" priority="1074">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:U4 AR4:XFD4">
+    <cfRule type="colorScale" priority="1080">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9928,8 +10367,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:XFD7">
-    <cfRule type="colorScale" priority="22">
+  <conditionalFormatting sqref="A6:U6 AR6:XFD6">
+    <cfRule type="colorScale" priority="1083">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9940,8 +10379,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A8:XFD8">
-    <cfRule type="colorScale" priority="23">
+  <conditionalFormatting sqref="A7:U7 AR7:XFD7">
+    <cfRule type="colorScale" priority="1086">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9952,8 +10391,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A9:XFD9">
-    <cfRule type="colorScale" priority="24">
+  <conditionalFormatting sqref="A8:U8 AR8:XFD8">
+    <cfRule type="colorScale" priority="1089">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9964,8 +10403,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A10:XFD10">
-    <cfRule type="colorScale" priority="25">
+  <conditionalFormatting sqref="A9:U9 AR9:XFD9">
+    <cfRule type="colorScale" priority="1092">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9976,8 +10415,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A24:XFD24 M26">
-    <cfRule type="colorScale" priority="26">
+  <conditionalFormatting sqref="A10:U10 AR10:XFD10">
+    <cfRule type="colorScale" priority="1095">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9988,8 +10427,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A34:XFD34">
-    <cfRule type="colorScale" priority="30">
+  <conditionalFormatting sqref="A24:U24 M26 X24 AR24:XFD24">
+    <cfRule type="colorScale" priority="1098">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10000,8 +10439,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A35:XFD35">
-    <cfRule type="colorScale" priority="27">
+  <conditionalFormatting sqref="A34:U34 AH34 AR34:XFD34">
+    <cfRule type="colorScale" priority="1102">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10012,8 +10451,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A38:XFD38">
-    <cfRule type="colorScale" priority="12">
+  <conditionalFormatting sqref="A35:U35 AI35 AR35:XFD35">
+    <cfRule type="colorScale" priority="1105">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10024,7 +10463,67 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A39:XFD39">
+  <conditionalFormatting sqref="A38:U38 AL38 AR38:XFD38">
+    <cfRule type="colorScale" priority="1108">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A39:U39 AM39 AR39:XFD39">
+    <cfRule type="colorScale" priority="1111">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7:U7">
+    <cfRule type="colorScale" priority="1196">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I8:R8 A8:G8 A6:E6 A4:C4 A2 J9:R9 A9:H9 K10:R10 A10:I10 A13:L13 A22:U22 AR34:XFD35 S8:U10 G6:U6 E4:U4 C2:U2 N13:U13 AR22:XFD22 A24:U24 AR13:XFD13 AR2:XFD2 AR4:XFD4 AR6:XFD6 AR8:XFD10 X24 AR24:XFD24 A34:U35">
+    <cfRule type="colorScale" priority="1199">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X24">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -10036,20 +10535,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="50">
+  <conditionalFormatting sqref="X24">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10060,7 +10547,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2">
+  <conditionalFormatting sqref="T21:T1048576 T2:T19">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S20:S1048576 S2:S18">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19 T20 X24">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -10072,208 +10583,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2 B26:Y26">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 B2:AQ2">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AN39:AQ39 B39:AL39 AM38:AQ38 B38:AK38 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 B26:Y26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2">
+  <conditionalFormatting sqref="X44:X1048576">
     <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AQ37 B40:AQ43">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B7:AQ7">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I8:XFD8 A8:G8 G6:XFD6 A6:E6 E4:XFD4 A4:C4 C2:XFD2 A2 J9:XFD9 A9:H9 K10:XFD10 A10:I10 N13:XFD13 A13:L13 W22:XFD22 A22:U22 Y24:XFD24 A24:W24 AI34:XFD34 A34:AG34 AJ35:XFD35 A35:AH35">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM39">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO40:AP40 AP41 O14:AK14 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 O19:R19 T21 T22:U22 T23:V23 T24:W24 Z27 Z28:AA28 Z29:AB29 Z30:AC30 Z31:AD31 Z32:AE32 Z33:AF33 Z34:AG34 Z35:AH35 Z36:AI36 Z37:AJ37 Z40:AM40 Z41:AN41 Z42:AO42 Z43:AP43 G8:G12 T25:X25 O20:S25 F2:L3 E4:F4 AQ14:AQ32 H7:K7 L7:L11 G4:L6 AM24:AP28 P15:AK15 Q16:AK16 R17:AK17 S18:AK18 T19:AK19 U20:AK20 V21:AK21 W22:AK22 X23:AK23 Y24:AL24 Z25:AL25 AA26:AL26 AB27:AL27 AC28:AL28 AD29:AP29 AE30:AP30 AF31:AP31 AG32:AP32 AQ34:AQ37 AH33:AQ33 AI34:AP34 AJ35:AP35 AK36:AP36 AL37:AP37 AQ40:AQ42 N13:AK13 M2:AQ12 AN13:AQ13 AN14:AP23 AL13:AM23 M15:N25 M14 H11:J11 H12:K12 H35:Y37 L24:L25 H24:K34 G24:G37 G13:L23 F7:F16 D6:E16 D17:F37 D5 B4:C37 L26:Y34 B40:Y43">
-    <cfRule type="colorScale" priority="220">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 D46:E46 B46 C45:E45 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 F45:M46 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N45:AQ56 AL57:AP67 O69:Y70 K60:N70">
-    <cfRule type="colorScale" priority="35">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 X24 W23 V22 U21 T20 S19 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2">
-    <cfRule type="colorScale" priority="48">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="49">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
-    <cfRule type="colorScale" priority="36">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="37">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AR43:XFD43 A43:AP43 AQ42:XFD42 A42:AO42 AP41:XFD41 A41:AN41 AO40:XFD40 A40:AM40 AL37:XFD37 A37:AJ37 AK36:XFD36 A36:AI36 AJ35:XFD35 A35:AH35 AI34:XFD34 A34:AG34 AH33:XFD33 A33:AF33 AG32:XFD32 A32:AE32 AF31:XFD31 A31:AD31 AE30:XFD30 A30:AC30 AD29:XFD29 A29:AB29 AC28:XFD28 A28:AA28 AB27:XFD27 A27:Z27 AA26:XFD26 Z25:XFD25 A25:X25 Y24:XFD24 A24:W24 X23:XFD23 A23:V23 W22:XFD22 A22:U22 V21:XFD21 A21:T21 U20:XFD20 A20:S20 T19:XFD19 A19:R19 S18:XFD18 A18:Q18 R17:XFD17 A17:P17 Q16:XFD16 A16:O16 P15:XFD15 A15:N15 O14:XFD14 A14:M14 N13:XFD13 A13:L13 M12:XFD12 A12:K12 L11:XFD11 A11:J11 K10:XFD10 A10:I10 J9:XFD9 A9:H9 I8:XFD8 A8:G8 H7:XFD7 A7:F7 G6:XFD6 A6:E6 F5:XFD5 A5:D5 E4:XFD4 A4:C4 D3:XFD3 A3:B3 C2:XFD2 A2 A26:Y26">
-    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10694,7 +11005,7 @@
         <v>43</v>
       </c>
       <c r="D18" s="33">
-        <f>'Influence Matrix'!B19</f>
+        <f>'Influence Matrix'!B20</f>
         <v>0</v>
       </c>
       <c r="G18" t="s">
@@ -10715,7 +11026,7 @@
         <v>19</v>
       </c>
       <c r="D19" s="24">
-        <f>'Influence Matrix'!B20</f>
+        <f>'Influence Matrix'!B19</f>
         <v>-0.06</v>
       </c>
       <c r="G19" t="s">
@@ -11462,7 +11773,7 @@
         <v>43</v>
       </c>
       <c r="D59" s="33">
-        <f>'Influence Matrix'!C19</f>
+        <f>'Influence Matrix'!C20</f>
         <v>-0.08</v>
       </c>
     </row>
@@ -11477,7 +11788,7 @@
         <v>19</v>
       </c>
       <c r="D60" s="33">
-        <f>'Influence Matrix'!C20</f>
+        <f>'Influence Matrix'!C19</f>
         <v>0.01</v>
       </c>
     </row>
@@ -11996,13 +12307,13 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>43</v>
+        <v>195</v>
       </c>
       <c r="B18" s="1"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="B19" s="1"/>
     </row>

</xml_diff>

<commit_message>
Finished edge: Agriculture → Firearms
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="683" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEA60180-11B0-4CD0-B55C-A8983EBB7449}"/>
+  <xr:revisionPtr revIDLastSave="686" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C340401B-1816-451D-A6E5-D123E6DE050E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -4396,7 +4396,7 @@
         <v>-0.06</v>
       </c>
       <c r="C19" s="12">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="D19" s="13">
         <v>-0.14000000000000001</v>
@@ -11789,7 +11789,7 @@
       </c>
       <c r="D60" s="33">
         <f>'Influence Matrix'!C19</f>
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added healthcare edges for Agriculture
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="686" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C340401B-1816-451D-A6E5-D123E6DE050E}"/>
+  <xr:revisionPtr revIDLastSave="693" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69B9EFBD-9BA7-422A-9028-30F9BF297802}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -4680,7 +4680,7 @@
         <v>-0.13</v>
       </c>
       <c r="C21" s="12">
-        <v>-0.13</v>
+        <v>0.06</v>
       </c>
       <c r="D21" s="13">
         <v>0.16</v>
@@ -4822,7 +4822,7 @@
         <v>0.32</v>
       </c>
       <c r="C22" s="12">
-        <v>0.11</v>
+        <v>0.05</v>
       </c>
       <c r="D22" s="13">
         <v>-0.1</v>
@@ -4964,7 +4964,7 @@
         <v>-0.15</v>
       </c>
       <c r="C23" s="12">
-        <v>-7.0000000000000007E-2</v>
+        <v>0.03</v>
       </c>
       <c r="D23" s="13">
         <v>0.13</v>
@@ -9819,518 +9819,6 @@
       <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
     </customSheetView>
   </customSheetViews>
-  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
-    <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
-    <cfRule type="colorScale" priority="81">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="69">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7">
-    <cfRule type="colorScale" priority="37">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
-    <cfRule type="colorScale" priority="40">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM39">
-    <cfRule type="colorScale" priority="35">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 B46 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 D46:M46 C45:G45 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N46:AQ56 AA45:AQ45 AL57:AP67 O69:Y70 K60:N70">
-    <cfRule type="colorScale" priority="66">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 V22 U21 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2 W23">
-    <cfRule type="colorScale" priority="79">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="80">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
-    <cfRule type="colorScale" priority="67">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="68">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T19 S20">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S19">
-    <cfRule type="colorScale" priority="29">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3:B1048576">
-    <cfRule type="colorScale" priority="27">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C4:C1048576 C2">
-    <cfRule type="colorScale" priority="26">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D5:D1048576 D2:D3">
-    <cfRule type="colorScale" priority="25">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E1048576 E2:E4">
-    <cfRule type="colorScale" priority="24">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F1048576 F2:F5">
-    <cfRule type="colorScale" priority="23">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G8:G1048576 G2:G6">
-    <cfRule type="colorScale" priority="22">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H1048576 H2:H7">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I10:I1048576 I2:I8">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11:J1048576 J2:J9">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K12:K1048576 K2:K10">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L13:L1048576 L2:L11">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M1048576 M2:M12">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N15:N1048576 N2:N13">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O16:O1048576 O2:O14">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P17:P1048576 P2:P15">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q18:Q1048576 Q2:Q16">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R19:R1048576 R2:R17">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T18 S44:S1048576 T20:T43">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S19 T44:T1048576 S21:S43">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U22:U1048576 U2:U20">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V44:V1048576">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T21:T25 T19 U19:U20 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 B19:R37 S20:S37 X24 U22:U25 T26:U37 B40:U43">
-    <cfRule type="colorScale" priority="357">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
-    <cfRule type="colorScale" priority="474">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 X24 U22:U43">
-    <cfRule type="colorScale" priority="597">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
-    <cfRule type="colorScale" priority="726">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T21:T25 B19:R19 O14:R14 S14:S18 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 G8:G12 F2:L3 E4:F4 H7:K7 L7:L11 G4:L6 P15:R15 Q16:R16 R17 T14:T19 U14:U20 N13:U13 M2:U12 M15:N18 M20:R25 M14 H11:J11 H12:K12 H35:R37 S20:S37 L24:L25 H24:K34 G24:G37 G13:L18 G20:L23 F7:F16 D6:E16 D17:F18 D5 B4:C18 B20:F37 L26:R34 X24 U22:U25 T26:U37 B40:U43">
-    <cfRule type="colorScale" priority="768">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AR40:XFD43 T21:T25 U20 T2:U19 S2:S18 A18:Q18 R17 A17:P17 Q16:R16 A16:O16 P15:R15 A15:N15 O14:R14 A14:M14 N13:R13 A13:L13 M12:R12 A12:K12 L11:R11 A11:J11 K10:R10 A10:I10 J9:R9 A9:H9 I8:R8 A8:G8 H7:R7 A7:F7 G6:R6 A6:E6 F5:R5 A5:D5 E4:R4 A4:C4 D3:R3 A3:B3 C2:R2 A2 A19:R37 S20:S37 X24 AR2:XFD37 U22:U25 T26:U37 A40:U43">
-    <cfRule type="colorScale" priority="950">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S21:S43 T20:T43 U19:U20 B19:R43 T2:U18 S2:S19 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 X24 U22:U43">
-    <cfRule type="colorScale" priority="1070">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A2:U2 AR2:XFD2">
     <cfRule type="colorScale" priority="1071">
       <colorScale>
@@ -10340,18 +9828,6 @@
         <color rgb="FF63BE7B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
-    <cfRule type="colorScale" priority="1074">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10487,8 +9963,56 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
-    <cfRule type="colorScale" priority="1190">
+  <conditionalFormatting sqref="B2">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B1048576">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="474">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="597">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10511,6 +10035,114 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C4:C1048576 C2">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D5:D1048576 D2:D3">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6:E1048576 E2:E4">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7:F1048576 F2:F5">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7">
+    <cfRule type="colorScale" priority="37">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8:G1048576 G2:G6">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9:H1048576 H2:H7">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I10:I1048576 I2:I8">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I8:R8 A8:G8 A6:E6 A4:C4 A2 J9:R9 A9:H9 K10:R10 A10:I10 A13:L13 A22:U22 AR34:XFD35 S8:U10 G6:U6 E4:U4 C2:U2 N13:U13 AR22:XFD22 A24:U24 AR13:XFD13 AR2:XFD2 AR4:XFD4 AR6:XFD6 AR8:XFD10 X24 AR24:XFD24 A34:U35">
     <cfRule type="colorScale" priority="1199">
       <colorScale>
@@ -10523,8 +10155,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X24">
-    <cfRule type="colorScale" priority="5">
+  <conditionalFormatting sqref="J11:J1048576 J2:J9">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10535,8 +10167,258 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X24">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="K12:K1048576 K2:K10">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L13:L1048576 L2:L11">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M14:M1048576 M2:M12">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N15:N1048576 N2:N13">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O16:O1048576 O2:O14">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P17:P1048576 P2:P15">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q18:Q1048576 Q2:Q16">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R19:R1048576 R2:R17">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S19 T44:T1048576 S21:S43">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19 T20 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19 T20 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S20 T19">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S20:S1048576 S2:S18">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S21:S43 T20:T43 U19:U20 B19:R43 T2:U18 S2:S19 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 X24 U22:U43">
+    <cfRule type="colorScale" priority="1070">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2:T18 S44:S1048576 T20:T43">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 X24">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 V22 U21 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2 W23">
+    <cfRule type="colorScale" priority="80">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="79">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T21:T25 B19:R19 O14:R14 S14:S18 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 G8:G12 F2:L3 E4:F4 H7:K7 L7:L11 G4:L6 P15:R15 Q16:R16 R17 T14:T19 U14:U20 N13:U13 M2:U12 M15:N18 M20:R25 M14 H11:J11 H12:K12 H35:R37 S20:S37 L24:L25 H24:K34 G24:G37 G13:L18 G20:L23 F7:F16 D6:E16 D17:F18 D5 B4:C18 B20:F37 L26:R34 X24 U22:U25 T26:U37 B40:U43">
+    <cfRule type="colorScale" priority="768">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T21:T25 T19 U19:U20 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 C2:R2 B19:R37 S20:S37 X24 U22:U25 T26:U37 B40:U43">
+    <cfRule type="colorScale" priority="357">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10559,8 +10441,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S20:S1048576 S2:S18">
-    <cfRule type="colorScale" priority="3">
+  <conditionalFormatting sqref="U22:U1048576 U2:U20">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10571,8 +10453,66 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 X24">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="V44:V1048576">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X24">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X44:X1048576">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK37 AQ43 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39 AL38">
+    <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10583,8 +10523,66 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X44:X1048576">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="AM39">
+    <cfRule type="colorScale" priority="35">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 B46 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 D46:M46 C45:G45 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N46:AQ56 AA45:AQ45 AL57:AP67 O69:Y70 K60:N70">
+    <cfRule type="colorScale" priority="66">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
+    <cfRule type="colorScale" priority="68">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="67">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
+    <cfRule type="colorScale" priority="1074">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR40:XFD43 T21:T25 U20 T2:U19 S2:S18 A18:Q18 R17 A17:P17 Q16:R16 A16:O16 P15:R15 A15:N15 O14:R14 A14:M14 N13:R13 A13:L13 M12:R12 A12:K12 L11:R11 A11:J11 K10:R10 A10:I10 J9:R9 A9:H9 I8:R8 A8:G8 H7:R7 A7:F7 G6:R6 A6:E6 F5:R5 A5:D5 E4:R4 A4:C4 D3:R3 A3:B3 C2:R2 A2 A19:R37 S20:S37 X24 AR2:XFD37 U22:U25 T26:U37 A40:U43">
+    <cfRule type="colorScale" priority="950">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -11804,7 +11802,7 @@
       </c>
       <c r="D61" s="33">
         <f>'Influence Matrix'!C21</f>
-        <v>-0.13</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -11819,7 +11817,7 @@
       </c>
       <c r="D62" s="33">
         <f>'Influence Matrix'!C22</f>
-        <v>0.11</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -11834,7 +11832,7 @@
       </c>
       <c r="D63" s="33">
         <f>'Influence Matrix'!C23</f>
-        <v>-7.0000000000000007E-2</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added edge: Agriculture → Homelessness
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="693" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69B9EFBD-9BA7-422A-9028-30F9BF297802}"/>
+  <xr:revisionPtr revIDLastSave="694" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5963ABE-F90A-439A-8209-7A9F17B0CCFD}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -5106,7 +5106,7 @@
         <v>0.18</v>
       </c>
       <c r="C24" s="12">
-        <v>7.0000000000000007E-2</v>
+        <v>-0.06</v>
       </c>
       <c r="D24" s="13">
         <v>-0.2</v>
@@ -11847,7 +11847,7 @@
       </c>
       <c r="D64" s="33">
         <f>'Influence Matrix'!C24</f>
-        <v>7.0000000000000007E-2</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added edge: Agriculture → Immigration
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="694" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5963ABE-F90A-439A-8209-7A9F17B0CCFD}"/>
+  <xr:revisionPtr revIDLastSave="695" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78B80047-AFEB-4E21-BC7E-6EAA040BFD85}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -5248,7 +5248,7 @@
         <v>-0.04</v>
       </c>
       <c r="C25" s="12">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
       <c r="D25" s="13">
         <v>-0.31</v>
@@ -11862,7 +11862,7 @@
       </c>
       <c r="D65" s="33">
         <f>'Influence Matrix'!C25</f>
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added edge: Agriculture → Infrastructure
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="695" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78B80047-AFEB-4E21-BC7E-6EAA040BFD85}"/>
+  <xr:revisionPtr revIDLastSave="696" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD605238-34BD-4B4A-A5AC-56DF2C5CE705}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -5390,7 +5390,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="12">
-        <v>0.38</v>
+        <v>0.17</v>
       </c>
       <c r="D26" s="13">
         <v>-0.15</v>
@@ -11877,7 +11877,7 @@
       </c>
       <c r="D66" s="33">
         <f>'Influence Matrix'!C26</f>
-        <v>0.38</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added edge: Agriculture → Innovation, Law Enforcement, Liberty
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="696" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD605238-34BD-4B4A-A5AC-56DF2C5CE705}"/>
+  <xr:revisionPtr revIDLastSave="699" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F06D5C8-EB16-4624-8B5B-638A836D6FF3}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -5532,7 +5532,7 @@
         <v>-0.16</v>
       </c>
       <c r="C27" s="12">
-        <v>0.33</v>
+        <v>0.15</v>
       </c>
       <c r="D27" s="13">
         <v>-0.16</v>
@@ -5674,7 +5674,7 @@
         <v>0.2</v>
       </c>
       <c r="C28" s="12">
-        <v>-0.09</v>
+        <v>0</v>
       </c>
       <c r="D28" s="13">
         <v>0.22</v>
@@ -5816,7 +5816,7 @@
         <v>-0.22</v>
       </c>
       <c r="C29" s="12">
-        <v>0.25</v>
+        <v>0.03</v>
       </c>
       <c r="D29" s="13">
         <v>-0.35</v>
@@ -11892,7 +11892,7 @@
       </c>
       <c r="D67" s="33">
         <f>'Influence Matrix'!C27</f>
-        <v>0.33</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -11907,7 +11907,7 @@
       </c>
       <c r="D68" s="33">
         <f>'Influence Matrix'!C28</f>
-        <v>-0.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -11922,7 +11922,7 @@
       </c>
       <c r="D69" s="33">
         <f>'Influence Matrix'!C29</f>
-        <v>0.25</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update Agriculture edges: Market Freedom, Mental Health
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="699" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F06D5C8-EB16-4624-8B5B-638A836D6FF3}"/>
+  <xr:revisionPtr revIDLastSave="701" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C7A688B-3522-426B-B518-536F0C7D39BB}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -5958,7 +5958,7 @@
         <v>-0.11</v>
       </c>
       <c r="C30" s="12">
-        <v>0.27</v>
+        <v>0</v>
       </c>
       <c r="D30" s="13">
         <v>-0.18</v>
@@ -6100,7 +6100,7 @@
         <v>-0.35</v>
       </c>
       <c r="C31" s="12">
-        <v>-0.15</v>
+        <v>-0.12</v>
       </c>
       <c r="D31" s="13">
         <v>-0.13</v>
@@ -9987,18 +9987,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="69">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
     <cfRule type="colorScale" priority="474">
       <colorScale>
@@ -10047,18 +10035,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 AH34 AI35">
-    <cfRule type="colorScale" priority="726">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D5:D1048576 D2:D3">
     <cfRule type="colorScale" priority="25">
       <colorScale>
@@ -10068,6 +10044,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10191,6 +10179,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="M14:M1048576 M2:M12">
     <cfRule type="colorScale" priority="16">
       <colorScale>
@@ -10275,8 +10275,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
-    <cfRule type="colorScale" priority="45">
+  <conditionalFormatting sqref="S19 T20 X24">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10284,18 +10284,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
-    <cfRule type="colorScale" priority="81">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10308,18 +10296,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S20 T19">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10359,8 +10335,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 X24">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="T19 S20">
+    <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10368,6 +10344,30 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10499,19 +10499,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK37 AQ43 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
-    <cfRule type="colorScale" priority="1190">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM39 AL38">
+  <conditionalFormatting sqref="AL38 AM39">
     <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="min"/>
@@ -10569,6 +10557,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
     <cfRule type="colorScale" priority="1074">
       <colorScale>
@@ -11937,7 +11937,7 @@
       </c>
       <c r="D70" s="33">
         <f>'Influence Matrix'!C30</f>
-        <v>0.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="D71" s="33">
         <f>'Influence Matrix'!C31</f>
-        <v>-0.15</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added Agriculture edges: Military, Minimum Wage
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="701" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C7A688B-3522-426B-B518-536F0C7D39BB}"/>
+  <xr:revisionPtr revIDLastSave="702" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE03F952-7A18-4F44-BA47-F4E15BE0D3A4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -6384,7 +6384,7 @@
         <v>0</v>
       </c>
       <c r="C33" s="12">
-        <v>0.28000000000000003</v>
+        <v>0</v>
       </c>
       <c r="D33" s="13">
         <v>-0.05</v>
@@ -11982,7 +11982,7 @@
       </c>
       <c r="D73" s="33">
         <f>'Influence Matrix'!C33</f>
-        <v>0.28000000000000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update Agriculture edges: Poverty
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="704" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53919216-260C-4FF5-BEF1-835526C9CAE0}"/>
+  <xr:revisionPtr revIDLastSave="705" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DE77E19-88AA-4BAE-BA07-0BF4BE86AC45}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -6668,7 +6668,7 @@
         <v>0.24</v>
       </c>
       <c r="C35" s="12">
-        <v>-0.24</v>
+        <v>-0.28000000000000003</v>
       </c>
       <c r="D35" s="13">
         <v>-0.03</v>
@@ -12012,7 +12012,7 @@
       </c>
       <c r="D75" s="33">
         <f>'Influence Matrix'!C35</f>
-        <v>-0.24</v>
+        <v>-0.28000000000000003</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update Agriculture edges: Rule of Law
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="705" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DE77E19-88AA-4BAE-BA07-0BF4BE86AC45}"/>
+  <xr:revisionPtr revIDLastSave="707" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB2D998B-A577-45C1-8EF2-246613E3AA84}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -6810,7 +6810,7 @@
         <v>-0.12</v>
       </c>
       <c r="C36" s="12">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="D36" s="13">
         <v>-0.23</v>
@@ -6952,7 +6952,7 @@
         <v>-0.17</v>
       </c>
       <c r="C37" s="12">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D37" s="13">
         <v>-0.16</v>
@@ -12027,7 +12027,7 @@
       </c>
       <c r="D76" s="33">
         <f>'Influence Matrix'!C36</f>
-        <v>0</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="D77" s="33">
         <f>'Influence Matrix'!C37</f>
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated Agriculture edge: Sickness/Disease
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="707" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB2D998B-A577-45C1-8EF2-246613E3AA84}"/>
+  <xr:revisionPtr revIDLastSave="709" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B0F356D-38D1-4A1B-9105-DD85FFC02886}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -7094,7 +7094,7 @@
         <v>0.32</v>
       </c>
       <c r="C38" s="12">
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
       <c r="D38" s="13">
         <v>0</v>
@@ -9987,6 +9987,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
     <cfRule type="colorScale" priority="474">
       <colorScale>
@@ -10035,6 +10047,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D5:D1048576 D2:D3">
     <cfRule type="colorScale" priority="25">
       <colorScale>
@@ -10044,18 +10068,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
-    <cfRule type="colorScale" priority="726">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10179,18 +10191,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="69">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="M14:M1048576 M2:M12">
     <cfRule type="colorScale" priority="16">
       <colorScale>
@@ -10275,8 +10275,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 X24">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="S19 T20 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10284,6 +10284,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19 T20 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10296,6 +10308,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S20 T19">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10335,8 +10359,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T19 S20">
-    <cfRule type="colorScale" priority="31">
+  <conditionalFormatting sqref="T20 S19 X24">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10344,30 +10368,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
-    <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
-    <cfRule type="colorScale" priority="81">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10499,7 +10499,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
+  <conditionalFormatting sqref="AK37 AQ43 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39 AL38">
     <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="min"/>
@@ -10557,18 +10569,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
-    <cfRule type="colorScale" priority="1190">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
     <cfRule type="colorScale" priority="1074">
       <colorScale>
@@ -12057,7 +12057,7 @@
       </c>
       <c r="D78" s="33">
         <f>'Influence Matrix'!C38</f>
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated Agriculture edge: Spirituality/God
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="709" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B0F356D-38D1-4A1B-9105-DD85FFC02886}"/>
+  <xr:revisionPtr revIDLastSave="710" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E996E8E-84F7-42AE-8AE7-A818DE937FFD}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -7236,7 +7236,7 @@
         <v>-0.18</v>
       </c>
       <c r="C39" s="12">
-        <v>0.27</v>
+        <v>0.25</v>
       </c>
       <c r="D39" s="13">
         <v>0.09</v>
@@ -12072,7 +12072,7 @@
       </c>
       <c r="D79" s="33">
         <f>'Influence Matrix'!C39</f>
-        <v>0.27</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated Agriculture edge: Taxes
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="710" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E996E8E-84F7-42AE-8AE7-A818DE937FFD}"/>
+  <xr:revisionPtr revIDLastSave="711" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3888544-DAC1-4B70-80AE-E28283EE8705}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -7378,7 +7378,7 @@
         <v>0</v>
       </c>
       <c r="C40" s="12">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="D40" s="13">
         <v>0.21</v>
@@ -9987,18 +9987,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="69">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
     <cfRule type="colorScale" priority="474">
       <colorScale>
@@ -10047,18 +10035,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 AH34 AI35">
-    <cfRule type="colorScale" priority="726">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D5:D1048576 D2:D3">
     <cfRule type="colorScale" priority="25">
       <colorScale>
@@ -10068,6 +10044,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10191,6 +10179,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="M14:M1048576 M2:M12">
     <cfRule type="colorScale" priority="16">
       <colorScale>
@@ -10275,8 +10275,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
-    <cfRule type="colorScale" priority="45">
+  <conditionalFormatting sqref="S19 T20 X24">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10284,18 +10284,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
-    <cfRule type="colorScale" priority="81">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10308,18 +10296,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S20 T19">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10359,8 +10335,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 X24">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="T19 S20">
+    <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10368,6 +10344,30 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10499,19 +10499,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK37 AQ43 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
-    <cfRule type="colorScale" priority="1190">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM39 AL38">
+  <conditionalFormatting sqref="AL38 AM39">
     <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="min"/>
@@ -10569,6 +10557,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
     <cfRule type="colorScale" priority="1074">
       <colorScale>
@@ -12087,7 +12087,7 @@
       </c>
       <c r="D80" s="33">
         <f>'Influence Matrix'!C40</f>
-        <v>0.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated edges for Agriculture: Technology
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="711" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3888544-DAC1-4B70-80AE-E28283EE8705}"/>
+  <xr:revisionPtr revIDLastSave="712" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD53B99B-2E96-4330-BA15-F34716B88BD2}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -7520,7 +7520,7 @@
         <v>0</v>
       </c>
       <c r="C41" s="12">
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
       <c r="D41" s="13">
         <v>0.16</v>
@@ -12102,7 +12102,7 @@
       </c>
       <c r="D81" s="33">
         <f>'Influence Matrix'!C41</f>
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated edges for Agriculture: Transportation, Welfare
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="712" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD53B99B-2E96-4330-BA15-F34716B88BD2}"/>
+  <xr:revisionPtr revIDLastSave="718" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4642BD3-797A-4AD0-8D12-07D305482F40}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -7662,7 +7662,7 @@
         <v>0</v>
       </c>
       <c r="C42" s="14">
-        <v>0.2</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="D42" s="13">
         <v>0.24</v>
@@ -7804,7 +7804,7 @@
         <v>0.16</v>
       </c>
       <c r="C43" s="13">
-        <v>0.18</v>
+        <v>-0.12</v>
       </c>
       <c r="D43" s="13">
         <v>0.14000000000000001</v>
@@ -12117,7 +12117,7 @@
       </c>
       <c r="D82" s="33">
         <f>'Influence Matrix'!C42</f>
-        <v>0.2</v>
+        <v>0.28999999999999998</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="D83" s="33">
         <f>'Influence Matrix'!C43</f>
-        <v>0.18</v>
+        <v>-0.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Uploaded Authoritarianism Links.txt files; Finished edge for Authoritarianism → Addiction
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="718" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4642BD3-797A-4AD0-8D12-07D305482F40}"/>
+  <xr:revisionPtr revIDLastSave="719" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{586B53DE-8F7A-4381-B1F3-48A0AD0792F3}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -1985,7 +1985,7 @@
         <v>0.05</v>
       </c>
       <c r="D2" s="11">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E2" s="11">
         <v>0</v>
@@ -9987,6 +9987,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
     <cfRule type="colorScale" priority="474">
       <colorScale>
@@ -10035,6 +10047,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D5:D1048576 D2:D3">
     <cfRule type="colorScale" priority="25">
       <colorScale>
@@ -10044,18 +10068,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
-    <cfRule type="colorScale" priority="726">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10179,18 +10191,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="69">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="M14:M1048576 M2:M12">
     <cfRule type="colorScale" priority="16">
       <colorScale>
@@ -10275,8 +10275,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 X24">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="S19 T20 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10284,6 +10284,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19 T20 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10296,6 +10308,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S20 T19">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10335,8 +10359,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T19 S20">
-    <cfRule type="colorScale" priority="31">
+  <conditionalFormatting sqref="T20 S19 X24">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10344,30 +10368,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
-    <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
-    <cfRule type="colorScale" priority="81">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10499,7 +10499,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
+  <conditionalFormatting sqref="AK37 AQ43 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39 AL38">
     <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="min"/>
@@ -10557,18 +10569,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
-    <cfRule type="colorScale" priority="1190">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
     <cfRule type="colorScale" priority="1074">
       <colorScale>

</xml_diff>

<commit_message>
Edges for Authoritarianism → Agriculture, Birthrate
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="719" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{586B53DE-8F7A-4381-B1F3-48A0AD0792F3}"/>
+  <xr:revisionPtr revIDLastSave="720" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBE2F925-5F97-4C15-8C23-F55F5307C65C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -2127,7 +2127,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="13">
-        <v>-0.15</v>
+        <v>-0.08</v>
       </c>
       <c r="E3" s="13">
         <v>0.05</v>
@@ -9987,18 +9987,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="69">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
     <cfRule type="colorScale" priority="474">
       <colorScale>
@@ -10047,18 +10035,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 AH34 AI35">
-    <cfRule type="colorScale" priority="726">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D5:D1048576 D2:D3">
     <cfRule type="colorScale" priority="25">
       <colorScale>
@@ -10068,6 +10044,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10191,6 +10179,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="M14:M1048576 M2:M12">
     <cfRule type="colorScale" priority="16">
       <colorScale>
@@ -10275,8 +10275,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
-    <cfRule type="colorScale" priority="45">
+  <conditionalFormatting sqref="S19 T20 X24">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10284,18 +10284,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
-    <cfRule type="colorScale" priority="81">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10308,18 +10296,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S20 T19">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10359,8 +10335,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 X24">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="T19 S20">
+    <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10368,6 +10344,30 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10499,19 +10499,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK37 AQ43 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
-    <cfRule type="colorScale" priority="1190">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM39 AL38">
+  <conditionalFormatting sqref="AL38 AM39">
     <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="min"/>
@@ -10569,6 +10557,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
     <cfRule type="colorScale" priority="1074">
       <colorScale>

</xml_diff>

<commit_message>
Edges for Authoritarianism → Corruption
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="720" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBE2F925-5F97-4C15-8C23-F55F5307C65C}"/>
+  <xr:revisionPtr revIDLastSave="721" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58B6F344-AB2F-4383-971C-4305DD2F33B7}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -2553,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="11">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="E6" s="11">
         <v>0</v>

</xml_diff>

<commit_message>
Finished edge for Authoritarianism → Discrimination
</commit_message>
<xml_diff>
--- a/data/Influence_Matrix/Influence Matrix.xlsx
+++ b/data/Influence_Matrix/Influence Matrix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396CB379E3A3AB8/Documents/Projects/Society_v1/data/Influence_Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="721" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58B6F344-AB2F-4383-971C-4305DD2F33B7}"/>
+  <xr:revisionPtr revIDLastSave="729" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8149C72-9E01-4EC8-AF85-560E3FB5BD6D}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
+    <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" activeTab="2" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
   <sheets>
     <sheet name="Influence Matrix" sheetId="1" r:id="rId1"/>
@@ -1204,19 +1204,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="slantDashDot">
-        <color rgb="FFC00000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1261,6 +1248,17 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="slantDashDot">
+        <color rgb="FFC00000"/>
+      </left>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -1357,17 +1355,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1381,7 +1373,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1394,7 +1386,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1426,6 +1418,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1482,10 +1480,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2123,7 +2117,7 @@
       <c r="B3" s="12">
         <v>-0.08</v>
       </c>
-      <c r="C3" s="44">
+      <c r="C3" s="42">
         <v>1</v>
       </c>
       <c r="D3" s="13">
@@ -2979,7 +2973,7 @@
         <v>-0.17</v>
       </c>
       <c r="D9" s="13">
-        <v>-0.13</v>
+        <v>0</v>
       </c>
       <c r="E9" s="13">
         <v>-0.02</v>
@@ -7796,7 +7790,7 @@
       <c r="BA42" s="2"/>
     </row>
     <row r="43" spans="1:53" ht="17.100000000000001" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="45" t="str">
+      <c r="A43" s="43" t="str">
         <f>Sliders!A42</f>
         <v>Welfare</v>
       </c>
@@ -9987,6 +9981,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B19:R43 T21:T43 T19 U19:U20 S20:S43 S2:U18 B18:Q18 R17 B17:P17 Q16:R16 B16:O16 P15:R15 B15:N15 O14:R14 B14:M14 N13:R13 B13:L13 M12:R12 B12:K12 L11:R11 B11:J11 K10:R10 B10:I10 J9:R9 B9:H9 I8:R8 B8:G8 H7:R7 B7:F7 G6:R6 B6:E6 F5:R5 B5:D5 E4:R4 B4:C4 D3:R3 B3 B2:R2 X24 U22:U43">
     <cfRule type="colorScale" priority="474">
       <colorScale>
@@ -10035,6 +10041,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 AH34 AI35">
+    <cfRule type="colorScale" priority="726">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D5:D1048576 D2:D3">
     <cfRule type="colorScale" priority="25">
       <colorScale>
@@ -10044,18 +10062,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 AH34 AI35">
-    <cfRule type="colorScale" priority="726">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10179,18 +10185,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="69">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="M14:M1048576 M2:M12">
     <cfRule type="colorScale" priority="16">
       <colorScale>
@@ -10275,8 +10269,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S19 T20 X24">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="S19 T20 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
+    <cfRule type="colorScale" priority="45">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10284,6 +10278,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S19 T20 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10296,6 +10302,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S20 T19">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10335,8 +10353,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T19 S20">
-    <cfRule type="colorScale" priority="31">
+  <conditionalFormatting sqref="T20 S19 X24">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10344,30 +10362,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43 W23">
-    <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20 S19 B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 U21 V22 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 W23">
-    <cfRule type="colorScale" priority="81">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10499,7 +10493,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
+  <conditionalFormatting sqref="AK37 AQ43 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
+    <cfRule type="colorScale" priority="1190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM39 AL38">
     <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="min"/>
@@ -10557,18 +10563,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AQ43 AK37 B2:U21 B22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 B23:U37 AJ36 AN40 AO41 B40:U43 AP42">
-    <cfRule type="colorScale" priority="1190">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="AQ43:XFD43 AK37 A2:U21 A22:V22 W23 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 A23:U37 AJ36 AR2:XFD37 AN40 AO41 A40:U43 AP42 AR40:XFD42">
     <cfRule type="colorScale" priority="1074">
       <colorScale>
@@ -10681,7 +10675,7 @@
       <c r="C3" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="33">
+      <c r="D3" s="31">
         <f>'Influence Matrix'!B4</f>
         <v>0</v>
       </c>
@@ -10726,7 +10720,7 @@
       <c r="C5" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="33">
+      <c r="D5" s="31">
         <f>'Influence Matrix'!B6</f>
         <v>0</v>
       </c>
@@ -10768,7 +10762,7 @@
       <c r="C7" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="31">
         <f>'Influence Matrix'!B8</f>
         <v>0.3</v>
       </c>
@@ -10810,7 +10804,7 @@
       <c r="C9" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="33">
+      <c r="D9" s="31">
         <f>'Influence Matrix'!B10</f>
         <v>0</v>
       </c>
@@ -10831,7 +10825,7 @@
       <c r="C10" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="31">
         <f>'Influence Matrix'!B11</f>
         <v>0</v>
       </c>
@@ -10873,7 +10867,7 @@
       <c r="C12" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="33">
+      <c r="D12" s="31">
         <f>'Influence Matrix'!B13</f>
         <v>0</v>
       </c>
@@ -10936,7 +10930,7 @@
       <c r="C15" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="33">
+      <c r="D15" s="31">
         <f>'Influence Matrix'!B16</f>
         <v>0</v>
       </c>
@@ -11002,7 +10996,7 @@
       <c r="C18" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="33">
+      <c r="D18" s="31">
         <f>'Influence Matrix'!B20</f>
         <v>0</v>
       </c>
@@ -11107,7 +11101,7 @@
       <c r="C23" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="33">
+      <c r="D23" s="31">
         <f>'Influence Matrix'!B24</f>
         <v>0.18</v>
       </c>
@@ -11149,7 +11143,7 @@
       <c r="C25" t="s">
         <v>8</v>
       </c>
-      <c r="D25" s="33">
+      <c r="D25" s="31">
         <f>'Influence Matrix'!B26</f>
         <v>0</v>
       </c>
@@ -11170,7 +11164,7 @@
       <c r="C26" t="s">
         <v>9</v>
       </c>
-      <c r="D26" s="33">
+      <c r="D26" s="31">
         <f>'Influence Matrix'!B27</f>
         <v>-0.16</v>
       </c>
@@ -11296,7 +11290,7 @@
       <c r="C32" t="s">
         <v>12</v>
       </c>
-      <c r="D32" s="33">
+      <c r="D32" s="31">
         <f>'Influence Matrix'!B33</f>
         <v>0</v>
       </c>
@@ -11317,7 +11311,7 @@
       <c r="C33" t="s">
         <v>13</v>
       </c>
-      <c r="D33" s="33">
+      <c r="D33" s="31">
         <f>'Influence Matrix'!B34</f>
         <v>0</v>
       </c>
@@ -11404,7 +11398,7 @@
       <c r="C37" t="s">
         <v>15</v>
       </c>
-      <c r="D37" s="33">
+      <c r="D37" s="31">
         <f>'Influence Matrix'!B38</f>
         <v>0.32</v>
       </c>
@@ -11446,7 +11440,7 @@
       <c r="C39" t="s">
         <v>17</v>
       </c>
-      <c r="D39" s="33">
+      <c r="D39" s="31">
         <f>'Influence Matrix'!B40</f>
         <v>0</v>
       </c>
@@ -11467,7 +11461,7 @@
       <c r="C40" t="s">
         <v>34</v>
       </c>
-      <c r="D40" s="33">
+      <c r="D40" s="31">
         <f>'Influence Matrix'!B41</f>
         <v>0</v>
       </c>
@@ -11488,7 +11482,7 @@
       <c r="C41" t="s">
         <v>24</v>
       </c>
-      <c r="D41" s="33">
+      <c r="D41" s="31">
         <f>'Influence Matrix'!B42</f>
         <v>0</v>
       </c>
@@ -11530,7 +11524,7 @@
       <c r="C43" t="s">
         <v>26</v>
       </c>
-      <c r="D43" s="33">
+      <c r="D43" s="31">
         <f>'Influence Matrix'!C2</f>
         <v>0.05</v>
       </c>
@@ -11545,7 +11539,7 @@
       <c r="C44" t="s">
         <v>38</v>
       </c>
-      <c r="D44" s="33">
+      <c r="D44" s="31">
         <f>'Influence Matrix'!C4</f>
         <v>0.1</v>
       </c>
@@ -11560,7 +11554,7 @@
       <c r="C45" t="s">
         <v>1</v>
       </c>
-      <c r="D45" s="33">
+      <c r="D45" s="31">
         <f>'Influence Matrix'!C5</f>
         <v>7.0000000000000007E-2</v>
       </c>
@@ -11575,7 +11569,7 @@
       <c r="C46" t="s">
         <v>2</v>
       </c>
-      <c r="D46" s="33">
+      <c r="D46" s="31">
         <f>'Influence Matrix'!C6</f>
         <v>0</v>
       </c>
@@ -11590,7 +11584,7 @@
       <c r="C47" t="s">
         <v>35</v>
       </c>
-      <c r="D47" s="33">
+      <c r="D47" s="31">
         <f>'Influence Matrix'!C7</f>
         <v>-0.12</v>
       </c>
@@ -11605,7 +11599,7 @@
       <c r="C48" t="s">
         <v>3</v>
       </c>
-      <c r="D48" s="33">
+      <c r="D48" s="31">
         <f>'Influence Matrix'!C8</f>
         <v>-0.14000000000000001</v>
       </c>
@@ -11620,7 +11614,7 @@
       <c r="C49" t="s">
         <v>4</v>
       </c>
-      <c r="D49" s="33">
+      <c r="D49" s="31">
         <f>'Influence Matrix'!C9</f>
         <v>-0.17</v>
       </c>
@@ -11635,7 +11629,7 @@
       <c r="C50" t="s">
         <v>46</v>
       </c>
-      <c r="D50" s="33">
+      <c r="D50" s="31">
         <f>'Influence Matrix'!C10</f>
         <v>0.1</v>
       </c>
@@ -11650,7 +11644,7 @@
       <c r="C51" t="s">
         <v>21</v>
       </c>
-      <c r="D51" s="33">
+      <c r="D51" s="31">
         <f>'Influence Matrix'!C11</f>
         <v>0</v>
       </c>
@@ -11665,7 +11659,7 @@
       <c r="C52" t="s">
         <v>30</v>
       </c>
-      <c r="D52" s="33">
+      <c r="D52" s="31">
         <f>'Influence Matrix'!C12</f>
         <v>0</v>
       </c>
@@ -11680,7 +11674,7 @@
       <c r="C53" t="s">
         <v>22</v>
       </c>
-      <c r="D53" s="33">
+      <c r="D53" s="31">
         <f>'Influence Matrix'!C13</f>
         <v>0</v>
       </c>
@@ -11695,7 +11689,7 @@
       <c r="C54" t="s">
         <v>23</v>
       </c>
-      <c r="D54" s="33">
+      <c r="D54" s="31">
         <f>'Influence Matrix'!C14</f>
         <v>0</v>
       </c>
@@ -11710,7 +11704,7 @@
       <c r="C55" t="s">
         <v>5</v>
       </c>
-      <c r="D55" s="33">
+      <c r="D55" s="31">
         <f>'Influence Matrix'!C15</f>
         <v>0.21</v>
       </c>
@@ -11725,7 +11719,7 @@
       <c r="C56" t="s">
         <v>36</v>
       </c>
-      <c r="D56" s="33">
+      <c r="D56" s="31">
         <f>'Influence Matrix'!C16</f>
         <v>0.18</v>
       </c>
@@ -11740,7 +11734,7 @@
       <c r="C57" t="s">
         <v>18</v>
       </c>
-      <c r="D57" s="33">
+      <c r="D57" s="31">
         <f>'Influence Matrix'!C17</f>
         <v>-0.09</v>
       </c>
@@ -11755,7 +11749,7 @@
       <c r="C58" t="s">
         <v>39</v>
       </c>
-      <c r="D58" s="33">
+      <c r="D58" s="31">
         <f>'Influence Matrix'!C18</f>
         <v>0.14000000000000001</v>
       </c>
@@ -11770,7 +11764,7 @@
       <c r="C59" t="s">
         <v>43</v>
       </c>
-      <c r="D59" s="33">
+      <c r="D59" s="31">
         <f>'Influence Matrix'!C20</f>
         <v>-0.08</v>
       </c>
@@ -11785,7 +11779,7 @@
       <c r="C60" t="s">
         <v>19</v>
       </c>
-      <c r="D60" s="33">
+      <c r="D60" s="31">
         <f>'Influence Matrix'!C19</f>
         <v>0.1</v>
       </c>
@@ -11800,7 +11794,7 @@
       <c r="C61" t="s">
         <v>31</v>
       </c>
-      <c r="D61" s="33">
+      <c r="D61" s="31">
         <f>'Influence Matrix'!C21</f>
         <v>0.06</v>
       </c>
@@ -11815,7 +11809,7 @@
       <c r="C62" t="s">
         <v>32</v>
       </c>
-      <c r="D62" s="33">
+      <c r="D62" s="31">
         <f>'Influence Matrix'!C22</f>
         <v>0.05</v>
       </c>
@@ -11830,7 +11824,7 @@
       <c r="C63" t="s">
         <v>33</v>
       </c>
-      <c r="D63" s="33">
+      <c r="D63" s="31">
         <f>'Influence Matrix'!C23</f>
         <v>0.03</v>
       </c>
@@ -11845,7 +11839,7 @@
       <c r="C64" t="s">
         <v>6</v>
       </c>
-      <c r="D64" s="33">
+      <c r="D64" s="31">
         <f>'Influence Matrix'!C24</f>
         <v>-0.06</v>
       </c>
@@ -11860,7 +11854,7 @@
       <c r="C65" t="s">
         <v>7</v>
       </c>
-      <c r="D65" s="33">
+      <c r="D65" s="31">
         <f>'Influence Matrix'!C25</f>
         <v>0.13</v>
       </c>
@@ -11875,7 +11869,7 @@
       <c r="C66" t="s">
         <v>8</v>
       </c>
-      <c r="D66" s="33">
+      <c r="D66" s="31">
         <f>'Influence Matrix'!C26</f>
         <v>0.17</v>
       </c>
@@ -11890,7 +11884,7 @@
       <c r="C67" t="s">
         <v>9</v>
       </c>
-      <c r="D67" s="33">
+      <c r="D67" s="31">
         <f>'Influence Matrix'!C27</f>
         <v>0.15</v>
       </c>
@@ -11905,7 +11899,7 @@
       <c r="C68" t="s">
         <v>148</v>
       </c>
-      <c r="D68" s="33">
+      <c r="D68" s="31">
         <f>'Influence Matrix'!C28</f>
         <v>0</v>
       </c>
@@ -11920,7 +11914,7 @@
       <c r="C69" t="s">
         <v>10</v>
       </c>
-      <c r="D69" s="33">
+      <c r="D69" s="31">
         <f>'Influence Matrix'!C29</f>
         <v>0.03</v>
       </c>
@@ -11935,7 +11929,7 @@
       <c r="C70" t="s">
         <v>20</v>
       </c>
-      <c r="D70" s="33">
+      <c r="D70" s="31">
         <f>'Influence Matrix'!C30</f>
         <v>0</v>
       </c>
@@ -11950,7 +11944,7 @@
       <c r="C71" t="s">
         <v>11</v>
       </c>
-      <c r="D71" s="33">
+      <c r="D71" s="31">
         <f>'Influence Matrix'!C31</f>
         <v>-0.12</v>
       </c>
@@ -11965,7 +11959,7 @@
       <c r="C72" t="s">
         <v>164</v>
       </c>
-      <c r="D72" s="33">
+      <c r="D72" s="31">
         <f>'Influence Matrix'!C32</f>
         <v>0</v>
       </c>
@@ -11980,7 +11974,7 @@
       <c r="C73" t="s">
         <v>12</v>
       </c>
-      <c r="D73" s="33">
+      <c r="D73" s="31">
         <f>'Influence Matrix'!C33</f>
         <v>0</v>
       </c>
@@ -11995,7 +11989,7 @@
       <c r="C74" t="s">
         <v>13</v>
       </c>
-      <c r="D74" s="33">
+      <c r="D74" s="31">
         <f>'Influence Matrix'!C34</f>
         <v>0.31</v>
       </c>
@@ -12010,7 +12004,7 @@
       <c r="C75" t="s">
         <v>25</v>
       </c>
-      <c r="D75" s="33">
+      <c r="D75" s="31">
         <f>'Influence Matrix'!C35</f>
         <v>-0.28000000000000003</v>
       </c>
@@ -12025,7 +12019,7 @@
       <c r="C76" t="s">
         <v>14</v>
       </c>
-      <c r="D76" s="33">
+      <c r="D76" s="31">
         <f>'Influence Matrix'!C36</f>
         <v>0.04</v>
       </c>
@@ -12040,7 +12034,7 @@
       <c r="C77" t="s">
         <v>29</v>
       </c>
-      <c r="D77" s="33">
+      <c r="D77" s="31">
         <f>'Influence Matrix'!C37</f>
         <v>0</v>
       </c>
@@ -12055,7 +12049,7 @@
       <c r="C78" t="s">
         <v>15</v>
       </c>
-      <c r="D78" s="33">
+      <c r="D78" s="31">
         <f>'Influence Matrix'!C38</f>
         <v>0.18</v>
       </c>
@@ -12070,7 +12064,7 @@
       <c r="C79" t="s">
         <v>45</v>
       </c>
-      <c r="D79" s="33">
+      <c r="D79" s="31">
         <f>'Influence Matrix'!C39</f>
         <v>0.25</v>
       </c>
@@ -12085,7 +12079,7 @@
       <c r="C80" t="s">
         <v>17</v>
       </c>
-      <c r="D80" s="33">
+      <c r="D80" s="31">
         <f>'Influence Matrix'!C40</f>
         <v>0</v>
       </c>
@@ -12100,7 +12094,7 @@
       <c r="C81" t="s">
         <v>34</v>
       </c>
-      <c r="D81" s="33">
+      <c r="D81" s="31">
         <f>'Influence Matrix'!C41</f>
         <v>0.18</v>
       </c>
@@ -12115,7 +12109,7 @@
       <c r="C82" t="s">
         <v>24</v>
       </c>
-      <c r="D82" s="33">
+      <c r="D82" s="31">
         <f>'Influence Matrix'!C42</f>
         <v>0.28999999999999998</v>
       </c>
@@ -12130,7 +12124,7 @@
       <c r="C83" t="s">
         <v>44</v>
       </c>
-      <c r="D83" s="33">
+      <c r="D83" s="31">
         <f>'Influence Matrix'!C43</f>
         <v>-0.12</v>
       </c>
@@ -12212,30 +12206,30 @@
         <v>1</v>
       </c>
       <c r="B4" s="1"/>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="53"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
-      <c r="M4" s="46"/>
+      <c r="D4" s="51"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="44"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="44"/>
     </row>
     <row r="5" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="1"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="55"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="53"/>
     </row>
     <row r="6" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>35</v>
       </c>
       <c r="B6" s="1"/>
-      <c r="C6" s="56"/>
-      <c r="D6" s="57"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="55"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
@@ -12426,26 +12420,26 @@
       <c r="A37" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B37" s="32"/>
-      <c r="C37" s="58" t="s">
+      <c r="B37" s="60"/>
+      <c r="C37" s="56" t="s">
         <v>170</v>
       </c>
-      <c r="D37" s="58"/>
-      <c r="E37" s="58"/>
-      <c r="F37" s="58"/>
-      <c r="G37" s="58"/>
+      <c r="D37" s="56"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
       <c r="H37" s="28"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="B38" s="31"/>
-      <c r="C38" s="58"/>
-      <c r="D38" s="58"/>
-      <c r="E38" s="58"/>
-      <c r="F38" s="58"/>
-      <c r="G38" s="58"/>
+      <c r="B38" s="59"/>
+      <c r="C38" s="56"/>
+      <c r="D38" s="56"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
       <c r="H38" s="28"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -12453,11 +12447,11 @@
         <v>17</v>
       </c>
       <c r="B39" s="25"/>
-      <c r="C39" s="58"/>
-      <c r="D39" s="58"/>
-      <c r="E39" s="58"/>
-      <c r="F39" s="58"/>
-      <c r="G39" s="58"/>
+      <c r="C39" s="56"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="56"/>
       <c r="H39" s="28"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -12465,11 +12459,11 @@
         <v>34</v>
       </c>
       <c r="B40" s="25"/>
-      <c r="C40" s="58"/>
-      <c r="D40" s="58"/>
-      <c r="E40" s="58"/>
-      <c r="F40" s="58"/>
-      <c r="G40" s="58"/>
+      <c r="C40" s="56"/>
+      <c r="D40" s="56"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="56"/>
       <c r="H40" s="28"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -12524,170 +12518,170 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="J2" s="50" t="s">
+      <c r="J2" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="K2" s="51"/>
+      <c r="K2" s="49"/>
     </row>
     <row r="3" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="60"/>
-      <c r="E3" s="43" t="s">
+      <c r="C3" s="58"/>
+      <c r="E3" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="J3" s="47" t="s">
+      <c r="J3" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="K3" s="49" t="s">
+      <c r="K3" s="47" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="E4" s="40" t="s">
+      <c r="C4" s="33"/>
+      <c r="E4" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="J4" s="48" t="s">
+      <c r="J4" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="49" t="s">
+      <c r="K4" s="47" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="37"/>
-      <c r="E5" s="41" t="s">
+      <c r="C5" s="35"/>
+      <c r="E5" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="J5" s="48" t="s">
+      <c r="J5" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="K5" s="49" t="s">
+      <c r="K5" s="47" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="6" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="39"/>
-      <c r="E6" s="41" t="s">
+      <c r="C6" s="37"/>
+      <c r="E6" s="39" t="s">
         <v>165</v>
       </c>
-      <c r="J6" s="48" t="s">
+      <c r="J6" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="49" t="s">
+      <c r="K6" s="47" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="39" t="s">
         <v>166</v>
       </c>
-      <c r="J7" s="48" t="s">
+      <c r="J7" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="49" t="s">
+      <c r="K7" s="47" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="E8" s="41" t="s">
+      <c r="E8" s="39" t="s">
         <v>167</v>
       </c>
-      <c r="J8" s="48" t="s">
+      <c r="J8" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="49" t="s">
+      <c r="K8" s="47" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="39" t="s">
         <v>168</v>
       </c>
-      <c r="J9" s="48" t="s">
+      <c r="J9" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="K9" s="49" t="s">
+      <c r="K9" s="47" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="39" t="s">
         <v>169</v>
       </c>
-      <c r="J10" s="48" t="s">
+      <c r="J10" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="K10" s="49" t="s">
+      <c r="K10" s="47" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="E11" s="41"/>
-      <c r="J11" s="48" t="s">
+      <c r="E11" s="39"/>
+      <c r="J11" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="K11" s="49" t="s">
+      <c r="K11" s="47" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="12" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E12" s="42"/>
-      <c r="J12" s="48" t="s">
+      <c r="E12" s="40"/>
+      <c r="J12" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="K12" s="49" t="s">
+      <c r="K12" s="47" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="J13" s="48" t="s">
+      <c r="J13" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="K13" s="49" t="s">
+      <c r="K13" s="47" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="J14" s="48" t="s">
+      <c r="J14" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="K14" s="49" t="s">
+      <c r="K14" s="47" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="J15" s="48" t="s">
+      <c r="J15" s="46" t="s">
         <v>172</v>
       </c>
-      <c r="K15" s="49" t="s">
+      <c r="K15" s="47" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="J16" s="48" t="s">
+      <c r="J16" s="46" t="s">
         <v>173</v>
       </c>
-      <c r="K16" s="49" t="s">
+      <c r="K16" s="47" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="17" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="J17" s="49" t="s">
+      <c r="J17" s="47" t="s">
         <v>174</v>
       </c>
-      <c r="K17" s="49" t="s">
+      <c r="K17" s="47" t="s">
         <v>176</v>
       </c>
     </row>

</xml_diff>